<commit_message>
Update Sales Data 12-3
Update Sales Data 12-3
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7935B1B0-8ACE-4CD1-A440-EBC28DCC8482}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98412EF7-A2ED-4CC0-9FB9-C9560B1E0714}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1467,12 +1467,18 @@
       <c r="A49" s="3">
         <v>45991</v>
       </c>
-      <c r="B49" s="6"/>
+      <c r="B49" s="6">
+        <v>167539.18999999986</v>
+      </c>
       <c r="C49" s="6">
         <v>233700.89000000019</v>
       </c>
-      <c r="D49" s="6"/>
-      <c r="E49" s="7"/>
+      <c r="D49" s="6">
+        <v>26296.86</v>
+      </c>
+      <c r="E49" s="7">
+        <v>0.157</v>
+      </c>
       <c r="F49" s="7"/>
     </row>
     <row r="50" spans="1:6">
@@ -2499,21 +2505,27 @@
         <v>0.95269999999999999</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="15.75">
+    <row r="49" spans="1:7" ht="15.75">
       <c r="A49" s="3">
         <v>45991</v>
       </c>
       <c r="B49" s="12">
         <v>799</v>
       </c>
+      <c r="C49">
+        <v>574</v>
+      </c>
       <c r="E49" s="3">
         <v>45991</v>
       </c>
       <c r="F49">
         <v>0.97319999999999995</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="15.75">
+      <c r="G49">
+        <v>0.97119999999999995</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="15.75">
       <c r="A50" s="3">
         <v>45998</v>
       </c>
@@ -2527,7 +2539,7 @@
         <v>0.92079999999999995</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="15.75">
+    <row r="51" spans="1:7" ht="15.75">
       <c r="A51" s="3">
         <v>46005</v>
       </c>
@@ -2541,7 +2553,7 @@
         <v>0.91149999999999998</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="15.75">
+    <row r="52" spans="1:7" ht="15.75">
       <c r="A52" s="3">
         <v>46012</v>
       </c>
@@ -2555,7 +2567,7 @@
         <v>0.96930000000000005</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="15.75">
+    <row r="53" spans="1:7" ht="15.75">
       <c r="A53" s="3">
         <v>46019</v>
       </c>

</xml_diff>

<commit_message>
Payroll and Staffing Data 12-10-2025
Updating sales and staffing data
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98412EF7-A2ED-4CC0-9FB9-C9560B1E0714}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6072E9F5-4D5F-4060-84A7-B661F285AF23}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1485,12 +1485,18 @@
       <c r="A50" s="3">
         <v>45998</v>
       </c>
-      <c r="B50" s="6"/>
+      <c r="B50" s="6">
+        <v>307765.18999999954</v>
+      </c>
       <c r="C50" s="6">
         <v>434505.2599999996</v>
       </c>
-      <c r="D50" s="6"/>
-      <c r="E50" s="7"/>
+      <c r="D50" s="6">
+        <v>39028.44</v>
+      </c>
+      <c r="E50" s="7">
+        <v>0.1268</v>
+      </c>
       <c r="F50" s="7"/>
     </row>
     <row r="51" spans="1:6">
@@ -2532,11 +2538,17 @@
       <c r="B50" s="12">
         <v>1628</v>
       </c>
+      <c r="C50">
+        <v>1148</v>
+      </c>
       <c r="E50" s="3">
         <v>45998</v>
       </c>
       <c r="F50">
         <v>0.92079999999999995</v>
+      </c>
+      <c r="G50">
+        <v>0.95509999999999995</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="15.75">

</xml_diff>

<commit_message>
Sales and Staffing Data 12-14-2025
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6072E9F5-4D5F-4060-84A7-B661F285AF23}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73F9A58A-1D89-45C7-B6EA-6AA0936B985F}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1503,12 +1503,18 @@
       <c r="A51" s="3">
         <v>46005</v>
       </c>
-      <c r="B51" s="6"/>
+      <c r="B51" s="6">
+        <v>354162.70999999868</v>
+      </c>
       <c r="C51" s="6">
         <v>445049.27999999956</v>
       </c>
-      <c r="D51" s="6"/>
-      <c r="E51" s="7"/>
+      <c r="D51" s="6">
+        <v>53963.23</v>
+      </c>
+      <c r="E51" s="7">
+        <v>0.15240000000000001</v>
+      </c>
       <c r="F51" s="7"/>
     </row>
     <row r="52" spans="1:6">
@@ -2558,11 +2564,17 @@
       <c r="B51" s="12">
         <v>1566</v>
       </c>
+      <c r="C51">
+        <v>1328</v>
+      </c>
       <c r="E51" s="3">
         <v>46005</v>
       </c>
       <c r="F51">
         <v>0.91149999999999998</v>
+      </c>
+      <c r="G51">
+        <v>0.91969999999999996</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="15.75">

</xml_diff>

<commit_message>
Update Data for 12-21-25
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73F9A58A-1D89-45C7-B6EA-6AA0936B985F}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DE900C4-46FA-445A-BB94-D1C0A7D2314F}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1521,12 +1521,18 @@
       <c r="A52" s="3">
         <v>46012</v>
       </c>
-      <c r="B52" s="6"/>
+      <c r="B52" s="6">
+        <v>239344.09999999998</v>
+      </c>
       <c r="C52" s="6">
         <v>245005.63000000009</v>
       </c>
-      <c r="D52" s="6"/>
-      <c r="E52" s="7"/>
+      <c r="D52" s="6">
+        <v>35499.43</v>
+      </c>
+      <c r="E52" s="7">
+        <v>0.14829999999999999</v>
+      </c>
       <c r="F52" s="7"/>
     </row>
     <row r="53" spans="1:6">
@@ -2584,11 +2590,17 @@
       <c r="B52" s="10">
         <v>918</v>
       </c>
+      <c r="C52">
+        <v>893</v>
+      </c>
       <c r="E52" s="3">
         <v>46012</v>
       </c>
       <c r="F52">
         <v>0.96930000000000005</v>
+      </c>
+      <c r="G52">
+        <v>0.96120000000000005</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="15.75">

</xml_diff>

<commit_message>
Update Sales and Staffing Charts
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DE900C4-46FA-445A-BB94-D1C0A7D2314F}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C66F3114-28C8-4AB2-BB4E-A00245A7894A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -82,7 +82,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,6 +127,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -149,7 +156,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -165,6 +172,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,7 +508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F816EB9-28A4-4EE2-B083-40DDC67AF2B4}">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="1"/>
@@ -1539,13 +1547,345 @@
       <c r="A53" s="3">
         <v>46019</v>
       </c>
-      <c r="B53" s="6"/>
+      <c r="B53" s="6">
+        <v>126326.15999999999</v>
+      </c>
       <c r="C53" s="6">
         <v>130961.07000000005</v>
       </c>
-      <c r="D53" s="6"/>
-      <c r="E53" s="7"/>
+      <c r="D53" s="6">
+        <v>24648.43</v>
+      </c>
+      <c r="E53" s="7">
+        <v>0.1951</v>
+      </c>
       <c r="F53" s="7"/>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="3">
+        <v>46026</v>
+      </c>
+      <c r="C54" s="13">
+        <v>182536.52999999997</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="3">
+        <v>46033</v>
+      </c>
+      <c r="C55" s="13">
+        <v>243076.1799999997</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="3">
+        <v>46040</v>
+      </c>
+      <c r="C56" s="13">
+        <v>278804.31999999972</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" s="3">
+        <v>46047</v>
+      </c>
+      <c r="C57" s="13">
+        <v>325526.04999999946</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" s="3">
+        <v>46054</v>
+      </c>
+      <c r="C58" s="13">
+        <v>310656.64999999967</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" s="3">
+        <v>46061</v>
+      </c>
+      <c r="C59" s="13">
+        <v>307344.53999999957</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" s="3">
+        <v>46068</v>
+      </c>
+      <c r="C60" s="13">
+        <v>327003.24000000022</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" s="3">
+        <v>46075</v>
+      </c>
+      <c r="C61" s="13">
+        <v>282217.79999999958</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" s="3">
+        <v>46082</v>
+      </c>
+      <c r="C62" s="13">
+        <v>406848.86999999994</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" s="3">
+        <v>46089</v>
+      </c>
+      <c r="C63" s="13">
+        <v>492946.42999999959</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" s="3">
+        <v>46096</v>
+      </c>
+      <c r="C64" s="13">
+        <v>468207.41000000003</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="3">
+        <v>46103</v>
+      </c>
+      <c r="C65" s="13">
+        <v>375603.12999999931</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" s="3">
+        <v>46110</v>
+      </c>
+      <c r="C66" s="13">
+        <v>340411.14000000025</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" s="3">
+        <v>46117</v>
+      </c>
+      <c r="C67" s="13">
+        <v>273530.54999999987</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="3">
+        <v>46124</v>
+      </c>
+      <c r="C68" s="13">
+        <v>390090.2900000001</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="3">
+        <v>46131</v>
+      </c>
+      <c r="C69" s="13">
+        <v>313611.45000000007</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="3">
+        <v>46138</v>
+      </c>
+      <c r="C70" s="13">
+        <v>352412.92999999953</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" s="3">
+        <v>46145</v>
+      </c>
+      <c r="C71" s="13">
+        <v>364950.25999999949</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" s="3">
+        <v>46152</v>
+      </c>
+      <c r="C72" s="13">
+        <v>425529.93000000058</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" s="3">
+        <v>46159</v>
+      </c>
+      <c r="C73" s="13">
+        <v>336398.62999999977</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" s="3">
+        <v>46166</v>
+      </c>
+      <c r="C74" s="13">
+        <v>308474.0399999998</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" s="3">
+        <v>46173</v>
+      </c>
+      <c r="C75" s="13">
+        <v>265417.39000000007</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="C76" s="13">
+        <v>370097.93999999989</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="C77" s="13">
+        <v>322732.31999999989</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="C78" s="13">
+        <v>317908.49999999983</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="C79" s="13">
+        <v>331006.54999999987</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="C80" s="13">
+        <v>241221.7500000002</v>
+      </c>
+    </row>
+    <row r="81" spans="3:3">
+      <c r="C81" s="13">
+        <v>258857.03999999975</v>
+      </c>
+    </row>
+    <row r="82" spans="3:3">
+      <c r="C82" s="13">
+        <v>307494.14999999956</v>
+      </c>
+    </row>
+    <row r="83" spans="3:3">
+      <c r="C83" s="13">
+        <v>291026.70999999985</v>
+      </c>
+    </row>
+    <row r="84" spans="3:3">
+      <c r="C84" s="13">
+        <v>293420.3499999998</v>
+      </c>
+    </row>
+    <row r="85" spans="3:3">
+      <c r="C85" s="13">
+        <v>289832.15999999968</v>
+      </c>
+    </row>
+    <row r="86" spans="3:3">
+      <c r="C86" s="13">
+        <v>337646.1199999997</v>
+      </c>
+    </row>
+    <row r="87" spans="3:3">
+      <c r="C87" s="13">
+        <v>377961.64999999956</v>
+      </c>
+    </row>
+    <row r="88" spans="3:3">
+      <c r="C88" s="13">
+        <v>336254.38999999972</v>
+      </c>
+    </row>
+    <row r="89" spans="3:3">
+      <c r="C89" s="13">
+        <v>307653.78999999957</v>
+      </c>
+    </row>
+    <row r="90" spans="3:3">
+      <c r="C90" s="13">
+        <v>478029.9800000001</v>
+      </c>
+    </row>
+    <row r="91" spans="3:3">
+      <c r="C91" s="13">
+        <v>358026.49</v>
+      </c>
+    </row>
+    <row r="92" spans="3:3">
+      <c r="C92" s="13">
+        <v>377543.97999999917</v>
+      </c>
+    </row>
+    <row r="93" spans="3:3">
+      <c r="C93" s="13">
+        <v>357141.31999999983</v>
+      </c>
+    </row>
+    <row r="94" spans="3:3">
+      <c r="C94" s="13">
+        <v>343271.64999999973</v>
+      </c>
+    </row>
+    <row r="95" spans="3:3">
+      <c r="C95" s="13">
+        <v>395964.53000000026</v>
+      </c>
+    </row>
+    <row r="96" spans="3:3">
+      <c r="C96" s="13">
+        <v>417034.32999999961</v>
+      </c>
+    </row>
+    <row r="97" spans="3:3">
+      <c r="C97" s="13">
+        <v>389381.13999999932</v>
+      </c>
+    </row>
+    <row r="98" spans="3:3">
+      <c r="C98" s="13">
+        <v>394153.5100000003</v>
+      </c>
+    </row>
+    <row r="99" spans="3:3">
+      <c r="C99" s="13">
+        <v>358939.24000000005</v>
+      </c>
+    </row>
+    <row r="100" spans="3:3">
+      <c r="C100" s="13">
+        <v>527012.11999999965</v>
+      </c>
+    </row>
+    <row r="101" spans="3:3">
+      <c r="C101" s="13">
+        <v>233700.89000000019</v>
+      </c>
+    </row>
+    <row r="102" spans="3:3">
+      <c r="C102" s="13">
+        <v>434505.2599999996</v>
+      </c>
+    </row>
+    <row r="103" spans="3:3">
+      <c r="C103" s="13">
+        <v>445049.27999999956</v>
+      </c>
+    </row>
+    <row r="104" spans="3:3">
+      <c r="C104" s="13">
+        <v>245005.63000000009</v>
+      </c>
+    </row>
+    <row r="105" spans="3:3">
+      <c r="C105" s="13">
+        <v>130961.07000000005</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1554,7 +1894,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AC1FE54-5241-4EDC-8539-E8BDF3481B66}">
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
@@ -2610,8 +2950,565 @@
       <c r="B53" s="10">
         <v>450</v>
       </c>
+      <c r="C53">
+        <v>441</v>
+      </c>
       <c r="E53" s="3">
         <v>46019</v>
+      </c>
+      <c r="F53">
+        <v>0.98580000000000001</v>
+      </c>
+      <c r="G53">
+        <v>0.95450000000000002</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" s="3">
+        <v>46026</v>
+      </c>
+      <c r="B54">
+        <v>615</v>
+      </c>
+      <c r="E54" s="3">
+        <v>46026</v>
+      </c>
+      <c r="F54">
+        <v>0.95940000000000003</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55" s="3">
+        <v>46033</v>
+      </c>
+      <c r="B55">
+        <v>686</v>
+      </c>
+      <c r="E55" s="3">
+        <v>46033</v>
+      </c>
+      <c r="F55">
+        <v>0.9899</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56" s="3">
+        <v>46040</v>
+      </c>
+      <c r="B56">
+        <v>733</v>
+      </c>
+      <c r="E56" s="3">
+        <v>46040</v>
+      </c>
+      <c r="F56">
+        <v>0.97989999999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57" s="3">
+        <v>46047</v>
+      </c>
+      <c r="B57">
+        <v>845</v>
+      </c>
+      <c r="E57" s="3">
+        <v>46047</v>
+      </c>
+      <c r="F57">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58" s="3">
+        <v>46054</v>
+      </c>
+      <c r="B58">
+        <v>1038</v>
+      </c>
+      <c r="E58" s="3">
+        <v>46054</v>
+      </c>
+      <c r="F58">
+        <v>0.97460000000000002</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="A59" s="3">
+        <v>46061</v>
+      </c>
+      <c r="B59">
+        <v>802</v>
+      </c>
+      <c r="E59" s="3">
+        <v>46061</v>
+      </c>
+      <c r="F59">
+        <v>0.97330000000000005</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="A60" s="3">
+        <v>46068</v>
+      </c>
+      <c r="B60">
+        <v>794</v>
+      </c>
+      <c r="E60" s="3">
+        <v>46068</v>
+      </c>
+      <c r="F60">
+        <v>0.98629999999999995</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
+      <c r="A61" s="3">
+        <v>46075</v>
+      </c>
+      <c r="B61">
+        <v>703</v>
+      </c>
+      <c r="E61" s="3">
+        <v>46075</v>
+      </c>
+      <c r="F61">
+        <v>0.98870000000000002</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
+      <c r="A62" s="3">
+        <v>46082</v>
+      </c>
+      <c r="B62">
+        <v>986</v>
+      </c>
+      <c r="E62" s="3">
+        <v>46082</v>
+      </c>
+      <c r="F62">
+        <v>0.97619999999999996</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
+      <c r="A63" s="3">
+        <v>46089</v>
+      </c>
+      <c r="B63">
+        <v>864</v>
+      </c>
+      <c r="E63" s="3">
+        <v>46089</v>
+      </c>
+      <c r="F63">
+        <v>0.98180000000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
+      <c r="A64" s="3">
+        <v>46096</v>
+      </c>
+      <c r="B64">
+        <v>781</v>
+      </c>
+      <c r="E64" s="3">
+        <v>46096</v>
+      </c>
+      <c r="F64">
+        <v>0.98360000000000003</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="3">
+        <v>46103</v>
+      </c>
+      <c r="B65">
+        <v>1010</v>
+      </c>
+      <c r="E65" s="3">
+        <v>46103</v>
+      </c>
+      <c r="F65">
+        <v>0.95730000000000004</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" s="3">
+        <v>46110</v>
+      </c>
+      <c r="B66">
+        <v>901</v>
+      </c>
+      <c r="E66" s="3">
+        <v>46110</v>
+      </c>
+      <c r="F66">
+        <v>0.97409999999999997</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" s="3">
+        <v>46117</v>
+      </c>
+      <c r="B67">
+        <v>875</v>
+      </c>
+      <c r="E67" s="3">
+        <v>46117</v>
+      </c>
+      <c r="F67">
+        <v>0.97550000000000003</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" s="3">
+        <v>46124</v>
+      </c>
+      <c r="B68">
+        <v>845</v>
+      </c>
+      <c r="E68" s="3">
+        <v>46124</v>
+      </c>
+      <c r="F68">
+        <v>0.95369999999999999</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" s="3">
+        <v>46131</v>
+      </c>
+      <c r="B69">
+        <v>728</v>
+      </c>
+      <c r="E69" s="3">
+        <v>46131</v>
+      </c>
+      <c r="F69">
+        <v>0.96419999999999995</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" s="3">
+        <v>46138</v>
+      </c>
+      <c r="B70">
+        <v>1036</v>
+      </c>
+      <c r="E70" s="3">
+        <v>46138</v>
+      </c>
+      <c r="F70">
+        <v>0.93930000000000002</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" s="3">
+        <v>46145</v>
+      </c>
+      <c r="B71">
+        <v>951</v>
+      </c>
+      <c r="E71" s="3">
+        <v>46145</v>
+      </c>
+      <c r="F71">
+        <v>0.94069999999999998</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" s="3">
+        <v>46152</v>
+      </c>
+      <c r="B72">
+        <v>939</v>
+      </c>
+      <c r="E72" s="3">
+        <v>46152</v>
+      </c>
+      <c r="F72">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" s="3">
+        <v>46159</v>
+      </c>
+      <c r="B73">
+        <v>897</v>
+      </c>
+      <c r="E73" s="3">
+        <v>46159</v>
+      </c>
+      <c r="F73">
+        <v>0.93989999999999996</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" s="3">
+        <v>46166</v>
+      </c>
+      <c r="B74">
+        <v>885</v>
+      </c>
+      <c r="E74" s="3">
+        <v>46166</v>
+      </c>
+      <c r="F74">
+        <v>0.95679999999999998</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="A75" s="3">
+        <v>46173</v>
+      </c>
+      <c r="B75">
+        <v>688</v>
+      </c>
+      <c r="E75" s="3">
+        <v>46173</v>
+      </c>
+      <c r="F75">
+        <v>0.96899999999999997</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="B76">
+        <v>884</v>
+      </c>
+      <c r="F76">
+        <v>0.91600000000000004</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="B77">
+        <v>745</v>
+      </c>
+      <c r="F77">
+        <v>0.92430000000000001</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="B78">
+        <v>668</v>
+      </c>
+      <c r="F78">
+        <v>0.96389999999999998</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="B79">
+        <v>763</v>
+      </c>
+      <c r="F79">
+        <v>0.96460000000000001</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="B80">
+        <v>497</v>
+      </c>
+      <c r="F80">
+        <v>0.97829999999999995</v>
+      </c>
+    </row>
+    <row r="81" spans="2:6">
+      <c r="B81">
+        <v>594</v>
+      </c>
+      <c r="F81">
+        <v>0.9738</v>
+      </c>
+    </row>
+    <row r="82" spans="2:6">
+      <c r="B82">
+        <v>693</v>
+      </c>
+      <c r="F82">
+        <v>0.97460000000000002</v>
+      </c>
+    </row>
+    <row r="83" spans="2:6">
+      <c r="B83">
+        <v>651</v>
+      </c>
+      <c r="F83">
+        <v>0.97160000000000002</v>
+      </c>
+    </row>
+    <row r="84" spans="2:6">
+      <c r="B84">
+        <v>633</v>
+      </c>
+      <c r="F84">
+        <v>0.95909999999999995</v>
+      </c>
+    </row>
+    <row r="85" spans="2:6">
+      <c r="B85">
+        <v>839</v>
+      </c>
+      <c r="F85">
+        <v>0.86850000000000005</v>
+      </c>
+    </row>
+    <row r="86" spans="2:6">
+      <c r="B86">
+        <v>978</v>
+      </c>
+      <c r="F86">
+        <v>0.9395</v>
+      </c>
+    </row>
+    <row r="87" spans="2:6">
+      <c r="B87">
+        <v>800</v>
+      </c>
+      <c r="F87">
+        <v>0.95920000000000005</v>
+      </c>
+    </row>
+    <row r="88" spans="2:6">
+      <c r="B88">
+        <v>756</v>
+      </c>
+      <c r="F88">
+        <v>0.97289999999999999</v>
+      </c>
+    </row>
+    <row r="89" spans="2:6">
+      <c r="B89">
+        <v>896</v>
+      </c>
+      <c r="F89">
+        <v>0.92749999999999999</v>
+      </c>
+    </row>
+    <row r="90" spans="2:6">
+      <c r="B90">
+        <v>1039</v>
+      </c>
+      <c r="F90">
+        <v>0.92679999999999996</v>
+      </c>
+    </row>
+    <row r="91" spans="2:6">
+      <c r="B91">
+        <v>1221</v>
+      </c>
+      <c r="F91">
+        <v>0.89119999999999999</v>
+      </c>
+    </row>
+    <row r="92" spans="2:6">
+      <c r="B92">
+        <v>925</v>
+      </c>
+      <c r="F92">
+        <v>0.93049999999999999</v>
+      </c>
+    </row>
+    <row r="93" spans="2:6">
+      <c r="B93">
+        <v>969</v>
+      </c>
+      <c r="F93">
+        <v>0.9264</v>
+      </c>
+    </row>
+    <row r="94" spans="2:6">
+      <c r="B94">
+        <v>927</v>
+      </c>
+      <c r="F94">
+        <v>0.94020000000000004</v>
+      </c>
+    </row>
+    <row r="95" spans="2:6">
+      <c r="B95">
+        <v>1140</v>
+      </c>
+      <c r="F95">
+        <v>0.88719999999999999</v>
+      </c>
+    </row>
+    <row r="96" spans="2:6">
+      <c r="B96">
+        <v>913</v>
+      </c>
+      <c r="F96">
+        <v>0.95099999999999996</v>
+      </c>
+    </row>
+    <row r="97" spans="2:6">
+      <c r="B97">
+        <v>946</v>
+      </c>
+      <c r="F97">
+        <v>0.95069999999999999</v>
+      </c>
+    </row>
+    <row r="98" spans="2:6">
+      <c r="B98">
+        <v>1021</v>
+      </c>
+      <c r="F98">
+        <v>0.95689999999999997</v>
+      </c>
+    </row>
+    <row r="99" spans="2:6">
+      <c r="B99">
+        <v>1174</v>
+      </c>
+      <c r="F99">
+        <v>0.87290000000000001</v>
+      </c>
+    </row>
+    <row r="100" spans="2:6">
+      <c r="B100">
+        <v>1148</v>
+      </c>
+      <c r="F100">
+        <v>0.95269999999999999</v>
+      </c>
+    </row>
+    <row r="101" spans="2:6">
+      <c r="B101">
+        <v>574</v>
+      </c>
+      <c r="F101">
+        <v>0.97119999999999995</v>
+      </c>
+    </row>
+    <row r="102" spans="2:6">
+      <c r="B102">
+        <v>1148</v>
+      </c>
+      <c r="F102">
+        <v>0.95509999999999995</v>
+      </c>
+    </row>
+    <row r="103" spans="2:6">
+      <c r="B103">
+        <v>1328</v>
+      </c>
+      <c r="F103">
+        <v>0.91969999999999996</v>
+      </c>
+    </row>
+    <row r="104" spans="2:6">
+      <c r="B104">
+        <v>893</v>
+      </c>
+      <c r="F104">
+        <v>0.96120000000000005</v>
+      </c>
+    </row>
+    <row r="105" spans="2:6">
+      <c r="B105">
+        <v>441</v>
+      </c>
+      <c r="F105">
+        <v>0.95450000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Sales and Staffing Charts.xlsx
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C66F3114-28C8-4AB2-BB4E-A00245A7894A}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A0AA2F3-E5BC-4A59-8E55-C16501F7C511}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1594,298 +1594,166 @@
       </c>
     </row>
     <row r="58" spans="1:6">
-      <c r="A58" s="3">
-        <v>46054</v>
-      </c>
-      <c r="C58" s="13">
-        <v>310656.64999999967</v>
-      </c>
+      <c r="A58" s="3"/>
+      <c r="C58" s="13"/>
     </row>
     <row r="59" spans="1:6">
-      <c r="A59" s="3">
-        <v>46061</v>
-      </c>
-      <c r="C59" s="13">
-        <v>307344.53999999957</v>
-      </c>
+      <c r="A59" s="3"/>
+      <c r="C59" s="13"/>
     </row>
     <row r="60" spans="1:6">
-      <c r="A60" s="3">
-        <v>46068</v>
-      </c>
-      <c r="C60" s="13">
-        <v>327003.24000000022</v>
-      </c>
+      <c r="A60" s="3"/>
+      <c r="C60" s="13"/>
     </row>
     <row r="61" spans="1:6">
-      <c r="A61" s="3">
-        <v>46075</v>
-      </c>
-      <c r="C61" s="13">
-        <v>282217.79999999958</v>
-      </c>
+      <c r="A61" s="3"/>
+      <c r="C61" s="13"/>
     </row>
     <row r="62" spans="1:6">
-      <c r="A62" s="3">
-        <v>46082</v>
-      </c>
-      <c r="C62" s="13">
-        <v>406848.86999999994</v>
-      </c>
+      <c r="A62" s="3"/>
+      <c r="C62" s="13"/>
     </row>
     <row r="63" spans="1:6">
-      <c r="A63" s="3">
-        <v>46089</v>
-      </c>
-      <c r="C63" s="13">
-        <v>492946.42999999959</v>
-      </c>
+      <c r="A63" s="3"/>
+      <c r="C63" s="13"/>
     </row>
     <row r="64" spans="1:6">
-      <c r="A64" s="3">
-        <v>46096</v>
-      </c>
-      <c r="C64" s="13">
-        <v>468207.41000000003</v>
-      </c>
+      <c r="A64" s="3"/>
+      <c r="C64" s="13"/>
     </row>
     <row r="65" spans="1:3">
-      <c r="A65" s="3">
-        <v>46103</v>
-      </c>
-      <c r="C65" s="13">
-        <v>375603.12999999931</v>
-      </c>
+      <c r="A65" s="3"/>
+      <c r="C65" s="13"/>
     </row>
     <row r="66" spans="1:3">
-      <c r="A66" s="3">
-        <v>46110</v>
-      </c>
-      <c r="C66" s="13">
-        <v>340411.14000000025</v>
-      </c>
+      <c r="A66" s="3"/>
+      <c r="C66" s="13"/>
     </row>
     <row r="67" spans="1:3">
-      <c r="A67" s="3">
-        <v>46117</v>
-      </c>
-      <c r="C67" s="13">
-        <v>273530.54999999987</v>
-      </c>
+      <c r="A67" s="3"/>
+      <c r="C67" s="13"/>
     </row>
     <row r="68" spans="1:3">
-      <c r="A68" s="3">
-        <v>46124</v>
-      </c>
-      <c r="C68" s="13">
-        <v>390090.2900000001</v>
-      </c>
+      <c r="A68" s="3"/>
+      <c r="C68" s="13"/>
     </row>
     <row r="69" spans="1:3">
-      <c r="A69" s="3">
-        <v>46131</v>
-      </c>
-      <c r="C69" s="13">
-        <v>313611.45000000007</v>
-      </c>
+      <c r="A69" s="3"/>
+      <c r="C69" s="13"/>
     </row>
     <row r="70" spans="1:3">
-      <c r="A70" s="3">
-        <v>46138</v>
-      </c>
-      <c r="C70" s="13">
-        <v>352412.92999999953</v>
-      </c>
+      <c r="A70" s="3"/>
+      <c r="C70" s="13"/>
     </row>
     <row r="71" spans="1:3">
-      <c r="A71" s="3">
-        <v>46145</v>
-      </c>
-      <c r="C71" s="13">
-        <v>364950.25999999949</v>
-      </c>
+      <c r="A71" s="3"/>
+      <c r="C71" s="13"/>
     </row>
     <row r="72" spans="1:3">
-      <c r="A72" s="3">
-        <v>46152</v>
-      </c>
-      <c r="C72" s="13">
-        <v>425529.93000000058</v>
-      </c>
+      <c r="A72" s="3"/>
+      <c r="C72" s="13"/>
     </row>
     <row r="73" spans="1:3">
-      <c r="A73" s="3">
-        <v>46159</v>
-      </c>
-      <c r="C73" s="13">
-        <v>336398.62999999977</v>
-      </c>
+      <c r="A73" s="3"/>
+      <c r="C73" s="13"/>
     </row>
     <row r="74" spans="1:3">
-      <c r="A74" s="3">
-        <v>46166</v>
-      </c>
-      <c r="C74" s="13">
-        <v>308474.0399999998</v>
-      </c>
+      <c r="A74" s="3"/>
+      <c r="C74" s="13"/>
     </row>
     <row r="75" spans="1:3">
-      <c r="A75" s="3">
-        <v>46173</v>
-      </c>
-      <c r="C75" s="13">
-        <v>265417.39000000007</v>
-      </c>
+      <c r="A75" s="3"/>
+      <c r="C75" s="13"/>
     </row>
     <row r="76" spans="1:3">
-      <c r="C76" s="13">
-        <v>370097.93999999989</v>
-      </c>
+      <c r="C76" s="13"/>
     </row>
     <row r="77" spans="1:3">
-      <c r="C77" s="13">
-        <v>322732.31999999989</v>
-      </c>
+      <c r="C77" s="13"/>
     </row>
     <row r="78" spans="1:3">
-      <c r="C78" s="13">
-        <v>317908.49999999983</v>
-      </c>
+      <c r="C78" s="13"/>
     </row>
     <row r="79" spans="1:3">
-      <c r="C79" s="13">
-        <v>331006.54999999987</v>
-      </c>
+      <c r="C79" s="13"/>
     </row>
     <row r="80" spans="1:3">
-      <c r="C80" s="13">
-        <v>241221.7500000002</v>
-      </c>
+      <c r="C80" s="13"/>
     </row>
     <row r="81" spans="3:3">
-      <c r="C81" s="13">
-        <v>258857.03999999975</v>
-      </c>
+      <c r="C81" s="13"/>
     </row>
     <row r="82" spans="3:3">
-      <c r="C82" s="13">
-        <v>307494.14999999956</v>
-      </c>
+      <c r="C82" s="13"/>
     </row>
     <row r="83" spans="3:3">
-      <c r="C83" s="13">
-        <v>291026.70999999985</v>
-      </c>
+      <c r="C83" s="13"/>
     </row>
     <row r="84" spans="3:3">
-      <c r="C84" s="13">
-        <v>293420.3499999998</v>
-      </c>
+      <c r="C84" s="13"/>
     </row>
     <row r="85" spans="3:3">
-      <c r="C85" s="13">
-        <v>289832.15999999968</v>
-      </c>
+      <c r="C85" s="13"/>
     </row>
     <row r="86" spans="3:3">
-      <c r="C86" s="13">
-        <v>337646.1199999997</v>
-      </c>
+      <c r="C86" s="13"/>
     </row>
     <row r="87" spans="3:3">
-      <c r="C87" s="13">
-        <v>377961.64999999956</v>
-      </c>
+      <c r="C87" s="13"/>
     </row>
     <row r="88" spans="3:3">
-      <c r="C88" s="13">
-        <v>336254.38999999972</v>
-      </c>
+      <c r="C88" s="13"/>
     </row>
     <row r="89" spans="3:3">
-      <c r="C89" s="13">
-        <v>307653.78999999957</v>
-      </c>
+      <c r="C89" s="13"/>
     </row>
     <row r="90" spans="3:3">
-      <c r="C90" s="13">
-        <v>478029.9800000001</v>
-      </c>
+      <c r="C90" s="13"/>
     </row>
     <row r="91" spans="3:3">
-      <c r="C91" s="13">
-        <v>358026.49</v>
-      </c>
+      <c r="C91" s="13"/>
     </row>
     <row r="92" spans="3:3">
-      <c r="C92" s="13">
-        <v>377543.97999999917</v>
-      </c>
+      <c r="C92" s="13"/>
     </row>
     <row r="93" spans="3:3">
-      <c r="C93" s="13">
-        <v>357141.31999999983</v>
-      </c>
+      <c r="C93" s="13"/>
     </row>
     <row r="94" spans="3:3">
-      <c r="C94" s="13">
-        <v>343271.64999999973</v>
-      </c>
+      <c r="C94" s="13"/>
     </row>
     <row r="95" spans="3:3">
-      <c r="C95" s="13">
-        <v>395964.53000000026</v>
-      </c>
+      <c r="C95" s="13"/>
     </row>
     <row r="96" spans="3:3">
-      <c r="C96" s="13">
-        <v>417034.32999999961</v>
-      </c>
+      <c r="C96" s="13"/>
     </row>
     <row r="97" spans="3:3">
-      <c r="C97" s="13">
-        <v>389381.13999999932</v>
-      </c>
+      <c r="C97" s="13"/>
     </row>
     <row r="98" spans="3:3">
-      <c r="C98" s="13">
-        <v>394153.5100000003</v>
-      </c>
+      <c r="C98" s="13"/>
     </row>
     <row r="99" spans="3:3">
-      <c r="C99" s="13">
-        <v>358939.24000000005</v>
-      </c>
+      <c r="C99" s="13"/>
     </row>
     <row r="100" spans="3:3">
-      <c r="C100" s="13">
-        <v>527012.11999999965</v>
-      </c>
+      <c r="C100" s="13"/>
     </row>
     <row r="101" spans="3:3">
-      <c r="C101" s="13">
-        <v>233700.89000000019</v>
-      </c>
+      <c r="C101" s="13"/>
     </row>
     <row r="102" spans="3:3">
-      <c r="C102" s="13">
-        <v>434505.2599999996</v>
-      </c>
+      <c r="C102" s="13"/>
     </row>
     <row r="103" spans="3:3">
-      <c r="C103" s="13">
-        <v>445049.27999999956</v>
-      </c>
+      <c r="C103" s="13"/>
     </row>
     <row r="104" spans="3:3">
-      <c r="C104" s="13">
-        <v>245005.63000000009</v>
-      </c>
+      <c r="C104" s="13"/>
     </row>
     <row r="105" spans="3:3">
-      <c r="C105" s="13">
-        <v>130961.07000000005</v>
-      </c>
+      <c r="C105" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Data Update WE 1-4-2026
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A0AA2F3-E5BC-4A59-8E55-C16501F7C511}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5ECE1377-32DC-4A9B-9702-6D6278131A62}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1565,8 +1565,17 @@
       <c r="A54" s="3">
         <v>46026</v>
       </c>
+      <c r="B54" s="6">
+        <v>154215.48000000001</v>
+      </c>
       <c r="C54" s="13">
         <v>182536.52999999997</v>
+      </c>
+      <c r="D54" s="6">
+        <v>22093.8</v>
+      </c>
+      <c r="E54" s="7">
+        <v>0.14330000000000001</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2838,11 +2847,17 @@
       <c r="B54">
         <v>615</v>
       </c>
+      <c r="C54">
+        <v>539</v>
+      </c>
       <c r="E54" s="3">
         <v>46026</v>
       </c>
       <c r="F54">
         <v>0.95940000000000003</v>
+      </c>
+      <c r="G54">
+        <v>0.8528</v>
       </c>
     </row>
     <row r="55" spans="1:7">

</xml_diff>

<commit_message>
Data Update Jan 14
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5ECE1377-32DC-4A9B-9702-6D6278131A62}"/>
+  <xr:revisionPtr revIDLastSave="91" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E76396C7-459D-417F-86FF-D8F9AE181B83}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -60,19 +60,19 @@
     <t>Week Ending (Shift Count)</t>
   </si>
   <si>
-    <t>2024 (Shift Count)</t>
-  </si>
-  <si>
     <t>2025 (Shift Count)</t>
   </si>
   <si>
     <t>Week Ending (Fill Rate)</t>
   </si>
   <si>
-    <t>2024 (Fill Rate)</t>
+    <t>2025 (Fill Rate)</t>
   </si>
   <si>
-    <t>2025 (Fill Rate)</t>
+    <t>2026 (Shift Count)</t>
+  </si>
+  <si>
+    <t>2026 (Fill Rate)</t>
   </si>
 </sst>
 </file>
@@ -1582,8 +1582,17 @@
       <c r="A55" s="3">
         <v>46033</v>
       </c>
+      <c r="B55" s="6">
+        <v>147041.63</v>
+      </c>
       <c r="C55" s="13">
         <v>243076.1799999997</v>
+      </c>
+      <c r="D55" s="6">
+        <v>11291.47</v>
+      </c>
+      <c r="E55" s="7">
+        <v>7.6799999999999993E-2</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -1788,13 +1797,13 @@
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>11</v>
@@ -2867,11 +2876,17 @@
       <c r="B55">
         <v>686</v>
       </c>
+      <c r="C55">
+        <v>529</v>
+      </c>
       <c r="E55" s="3">
         <v>46033</v>
       </c>
       <c r="F55">
         <v>0.9899</v>
+      </c>
+      <c r="G55">
+        <v>0.98880000000000001</v>
       </c>
     </row>
     <row r="56" spans="1:7">

</xml_diff>

<commit_message>
Add Active Staff Workbook
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="95" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B84C57F0-9462-4C33-A0B2-2EC59B8F3CD0}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7075C14-94C6-4588-8ABA-28F3F0A4346C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
     <sheet name="Shift Count" sheetId="2" r:id="rId2"/>
+    <sheet name="Active Staff" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>2025 Revenue</t>
   </si>
@@ -74,6 +75,18 @@
   <si>
     <t>2024 (Shift Count)</t>
   </si>
+  <si>
+    <t>Active Staff</t>
+  </si>
+  <si>
+    <t>Worked</t>
+  </si>
+  <si>
+    <t>Percentage of Active Staff Working</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
 </sst>
 </file>
 
@@ -82,7 +95,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,6 +147,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -156,7 +175,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -173,6 +192,8 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3412,4 +3433,1054 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
+  <dimension ref="A1:D69"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="3">
+        <v>45571</v>
+      </c>
+      <c r="B2">
+        <v>2507</v>
+      </c>
+      <c r="C2">
+        <v>476</v>
+      </c>
+      <c r="D2" s="14">
+        <f>C2/B2</f>
+        <v>0.18986836856800957</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="3">
+        <v>45578</v>
+      </c>
+      <c r="B3">
+        <v>2485</v>
+      </c>
+      <c r="C3">
+        <v>445</v>
+      </c>
+      <c r="D3" s="14">
+        <f>C3/B3</f>
+        <v>0.17907444668008049</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="3">
+        <v>45585</v>
+      </c>
+      <c r="B4">
+        <v>2406</v>
+      </c>
+      <c r="C4">
+        <v>485</v>
+      </c>
+      <c r="D4" s="14">
+        <f>C4/B4</f>
+        <v>0.20157938487115545</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="3">
+        <v>45592</v>
+      </c>
+      <c r="B5">
+        <v>2178</v>
+      </c>
+      <c r="C5">
+        <v>515</v>
+      </c>
+      <c r="D5" s="14">
+        <f>C5/B5</f>
+        <v>0.23645546372819101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="3">
+        <v>45599</v>
+      </c>
+      <c r="B6">
+        <v>2069</v>
+      </c>
+      <c r="C6">
+        <v>516</v>
+      </c>
+      <c r="D6" s="14">
+        <f>C6/B6</f>
+        <v>0.24939584340260995</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="3">
+        <v>45606</v>
+      </c>
+      <c r="B7">
+        <v>2006</v>
+      </c>
+      <c r="C7">
+        <v>503</v>
+      </c>
+      <c r="D7" s="14">
+        <f>C7/B7</f>
+        <v>0.25074775672981059</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="3">
+        <v>45613</v>
+      </c>
+      <c r="B8">
+        <v>1959</v>
+      </c>
+      <c r="C8">
+        <v>455</v>
+      </c>
+      <c r="D8" s="14">
+        <f>C8/B8</f>
+        <v>0.23226135783563043</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="3">
+        <v>45620</v>
+      </c>
+      <c r="B9">
+        <v>1896</v>
+      </c>
+      <c r="C9">
+        <v>715</v>
+      </c>
+      <c r="D9" s="14">
+        <f>C9/B9</f>
+        <v>0.37710970464135019</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="3">
+        <v>45627</v>
+      </c>
+      <c r="B10">
+        <v>1908</v>
+      </c>
+      <c r="C10">
+        <v>348</v>
+      </c>
+      <c r="D10" s="14">
+        <f>C10/B10</f>
+        <v>0.18238993710691823</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="3">
+        <v>45634</v>
+      </c>
+      <c r="B11">
+        <v>1837</v>
+      </c>
+      <c r="C11">
+        <v>661</v>
+      </c>
+      <c r="D11" s="14">
+        <f>C11/B11</f>
+        <v>0.35982580293957539</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="3">
+        <v>45641</v>
+      </c>
+      <c r="B12">
+        <v>1769</v>
+      </c>
+      <c r="C12">
+        <v>557</v>
+      </c>
+      <c r="D12" s="14">
+        <f>C12/B12</f>
+        <v>0.31486715658564163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="3">
+        <v>45648</v>
+      </c>
+      <c r="B13">
+        <v>1675</v>
+      </c>
+      <c r="C13">
+        <v>380</v>
+      </c>
+      <c r="D13" s="14">
+        <f>C13/B13</f>
+        <v>0.22686567164179106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="3">
+        <v>45655</v>
+      </c>
+      <c r="B14">
+        <v>1590</v>
+      </c>
+      <c r="C14">
+        <v>210</v>
+      </c>
+      <c r="D14" s="14">
+        <f>C14/B14</f>
+        <v>0.13207547169811321</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="3">
+        <v>45662</v>
+      </c>
+      <c r="B15">
+        <v>1562</v>
+      </c>
+      <c r="C15">
+        <v>279</v>
+      </c>
+      <c r="D15" s="14">
+        <f>C15/B15</f>
+        <v>0.17861715749039692</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="3">
+        <v>45669</v>
+      </c>
+      <c r="B16">
+        <v>1537</v>
+      </c>
+      <c r="C16">
+        <v>269</v>
+      </c>
+      <c r="D16" s="14">
+        <f>C16/B16</f>
+        <v>0.17501626545217958</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="3">
+        <v>45676</v>
+      </c>
+      <c r="B17">
+        <v>1541</v>
+      </c>
+      <c r="C17">
+        <v>272</v>
+      </c>
+      <c r="D17" s="14">
+        <f>C17/B17</f>
+        <v>0.17650876054510059</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="3">
+        <v>45683</v>
+      </c>
+      <c r="B18">
+        <v>1507</v>
+      </c>
+      <c r="C18">
+        <v>321</v>
+      </c>
+      <c r="D18" s="14">
+        <f>C18/B18</f>
+        <v>0.21300597213005973</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="3">
+        <v>45690</v>
+      </c>
+      <c r="B19">
+        <v>1425</v>
+      </c>
+      <c r="C19">
+        <v>413</v>
+      </c>
+      <c r="D19" s="14">
+        <f>C19/B19</f>
+        <v>0.28982456140350876</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="3">
+        <v>45697</v>
+      </c>
+      <c r="B20">
+        <v>1421</v>
+      </c>
+      <c r="C20">
+        <v>249</v>
+      </c>
+      <c r="D20" s="14">
+        <f>C20/B20</f>
+        <v>0.17522871217452499</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="3">
+        <v>45704</v>
+      </c>
+      <c r="B21">
+        <v>1292</v>
+      </c>
+      <c r="C21">
+        <v>301</v>
+      </c>
+      <c r="D21" s="14">
+        <f>C21/B21</f>
+        <v>0.23297213622291021</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="3">
+        <v>45711</v>
+      </c>
+      <c r="B22">
+        <v>1300</v>
+      </c>
+      <c r="C22">
+        <v>294</v>
+      </c>
+      <c r="D22" s="14">
+        <f>C22/B22</f>
+        <v>0.22615384615384615</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="3">
+        <v>45718</v>
+      </c>
+      <c r="B23">
+        <v>1330</v>
+      </c>
+      <c r="C23">
+        <v>361</v>
+      </c>
+      <c r="D23" s="14">
+        <f>C23/B23</f>
+        <v>0.27142857142857141</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="3">
+        <v>45725</v>
+      </c>
+      <c r="B24">
+        <v>1359</v>
+      </c>
+      <c r="C24">
+        <v>361</v>
+      </c>
+      <c r="D24" s="14">
+        <f>C24/B24</f>
+        <v>0.2656364974245769</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="3">
+        <v>45732</v>
+      </c>
+      <c r="B25">
+        <v>1343</v>
+      </c>
+      <c r="C25">
+        <v>293</v>
+      </c>
+      <c r="D25" s="14">
+        <f>C25/B25</f>
+        <v>0.21816827997021593</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="3">
+        <v>45739</v>
+      </c>
+      <c r="B26">
+        <v>1312</v>
+      </c>
+      <c r="C26">
+        <v>360</v>
+      </c>
+      <c r="D26" s="14">
+        <f>C26/B26</f>
+        <v>0.27439024390243905</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="3">
+        <v>45746</v>
+      </c>
+      <c r="B27">
+        <v>1333</v>
+      </c>
+      <c r="C27">
+        <v>319</v>
+      </c>
+      <c r="D27" s="14">
+        <f>C27/B27</f>
+        <v>0.23930982745686422</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="3">
+        <v>45753</v>
+      </c>
+      <c r="B28">
+        <v>1250</v>
+      </c>
+      <c r="C28">
+        <v>340</v>
+      </c>
+      <c r="D28" s="14">
+        <f>C28/B28</f>
+        <v>0.27200000000000002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="3">
+        <v>45760</v>
+      </c>
+      <c r="B29">
+        <v>1225</v>
+      </c>
+      <c r="C29">
+        <v>311</v>
+      </c>
+      <c r="D29" s="14">
+        <f>C29/B29</f>
+        <v>0.25387755102040815</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="3">
+        <v>45767</v>
+      </c>
+      <c r="B30">
+        <v>1186</v>
+      </c>
+      <c r="C30">
+        <v>274</v>
+      </c>
+      <c r="D30" s="14">
+        <f>C30/B30</f>
+        <v>0.23102866779089376</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="3">
+        <v>45774</v>
+      </c>
+      <c r="B31">
+        <v>1156</v>
+      </c>
+      <c r="C31">
+        <v>405</v>
+      </c>
+      <c r="D31" s="14">
+        <f>C31/B31</f>
+        <v>0.35034602076124566</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="3">
+        <v>45781</v>
+      </c>
+      <c r="B32">
+        <v>1163</v>
+      </c>
+      <c r="C32">
+        <v>384</v>
+      </c>
+      <c r="D32" s="14">
+        <f>C32/B32</f>
+        <v>0.33018056749785041</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="3">
+        <v>45788</v>
+      </c>
+      <c r="B33">
+        <v>1145</v>
+      </c>
+      <c r="C33">
+        <v>380</v>
+      </c>
+      <c r="D33" s="14">
+        <f>C33/B33</f>
+        <v>0.33187772925764192</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="3">
+        <v>45795</v>
+      </c>
+      <c r="B34">
+        <v>1145</v>
+      </c>
+      <c r="C34">
+        <v>363</v>
+      </c>
+      <c r="D34" s="14">
+        <f>C34/B34</f>
+        <v>0.31703056768558951</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="3">
+        <v>45802</v>
+      </c>
+      <c r="B35">
+        <v>1134</v>
+      </c>
+      <c r="C35">
+        <v>342</v>
+      </c>
+      <c r="D35" s="14">
+        <f>C35/B35</f>
+        <v>0.30158730158730157</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="3">
+        <v>45809</v>
+      </c>
+      <c r="B36">
+        <v>1118</v>
+      </c>
+      <c r="C36">
+        <v>293</v>
+      </c>
+      <c r="D36" s="14">
+        <f>C36/B36</f>
+        <v>0.26207513416815742</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="3">
+        <v>45816</v>
+      </c>
+      <c r="B37">
+        <v>1115</v>
+      </c>
+      <c r="C37">
+        <v>375</v>
+      </c>
+      <c r="D37" s="14">
+        <f>C37/B37</f>
+        <v>0.33632286995515698</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="3">
+        <v>45823</v>
+      </c>
+      <c r="B38">
+        <v>1130</v>
+      </c>
+      <c r="C38">
+        <v>288</v>
+      </c>
+      <c r="D38" s="14">
+        <f>C38/B38</f>
+        <v>0.25486725663716814</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="3">
+        <v>45830</v>
+      </c>
+      <c r="B39" s="15">
+        <v>1105</v>
+      </c>
+      <c r="C39" s="15">
+        <v>257</v>
+      </c>
+      <c r="D39" s="14">
+        <f>C39/B39</f>
+        <v>0.232579185520362</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="3">
+        <v>45837</v>
+      </c>
+      <c r="B40" s="15">
+        <v>1123</v>
+      </c>
+      <c r="C40" s="15">
+        <v>273</v>
+      </c>
+      <c r="D40" s="14">
+        <f>C40/B40</f>
+        <v>0.24309884238646481</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="3">
+        <v>45844</v>
+      </c>
+      <c r="B41">
+        <v>1097</v>
+      </c>
+      <c r="C41">
+        <v>198</v>
+      </c>
+      <c r="D41" s="14">
+        <f>C41/B41</f>
+        <v>0.18049225159525981</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="3">
+        <v>45851</v>
+      </c>
+      <c r="B42">
+        <v>1062</v>
+      </c>
+      <c r="C42">
+        <v>216</v>
+      </c>
+      <c r="D42" s="14">
+        <f>C42/B42</f>
+        <v>0.20338983050847459</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="3">
+        <v>45858</v>
+      </c>
+      <c r="B43">
+        <v>1047</v>
+      </c>
+      <c r="C43">
+        <v>247</v>
+      </c>
+      <c r="D43" s="14">
+        <f>C43/B43</f>
+        <v>0.23591212989493793</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="3">
+        <v>45865</v>
+      </c>
+      <c r="B44">
+        <v>1015</v>
+      </c>
+      <c r="C44">
+        <v>215</v>
+      </c>
+      <c r="D44" s="14">
+        <f>C44/B44</f>
+        <v>0.21182266009852216</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="3">
+        <v>45872</v>
+      </c>
+      <c r="B45">
+        <v>982</v>
+      </c>
+      <c r="C45">
+        <v>214</v>
+      </c>
+      <c r="D45" s="14">
+        <f>C45/B45</f>
+        <v>0.21792260692464357</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="3">
+        <v>45879</v>
+      </c>
+      <c r="B46">
+        <v>965</v>
+      </c>
+      <c r="C46">
+        <v>356</v>
+      </c>
+      <c r="D46" s="14">
+        <f>C46/B46</f>
+        <v>0.36891191709844562</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="3">
+        <v>45886</v>
+      </c>
+      <c r="B47">
+        <v>958</v>
+      </c>
+      <c r="C47">
+        <v>387</v>
+      </c>
+      <c r="D47" s="14">
+        <f>C47/B47</f>
+        <v>0.40396659707724425</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="3">
+        <v>45893</v>
+      </c>
+      <c r="B48">
+        <v>1034</v>
+      </c>
+      <c r="C48">
+        <v>284</v>
+      </c>
+      <c r="D48" s="14">
+        <f>C48/B48</f>
+        <v>0.27466150870406192</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="3">
+        <v>45900</v>
+      </c>
+      <c r="B49">
+        <v>1025</v>
+      </c>
+      <c r="C49">
+        <v>274</v>
+      </c>
+      <c r="D49" s="14">
+        <f>C49/B49</f>
+        <v>0.26731707317073172</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="3">
+        <v>45907</v>
+      </c>
+      <c r="B50">
+        <v>1021</v>
+      </c>
+      <c r="C50">
+        <v>365</v>
+      </c>
+      <c r="D50" s="14">
+        <f>C50/B50</f>
+        <v>0.3574926542605289</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="3">
+        <v>45914</v>
+      </c>
+      <c r="B51">
+        <v>1004</v>
+      </c>
+      <c r="C51">
+        <v>380</v>
+      </c>
+      <c r="D51" s="14">
+        <f>C51/B51</f>
+        <v>0.37848605577689243</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="3">
+        <v>45921</v>
+      </c>
+      <c r="B52">
+        <v>1023</v>
+      </c>
+      <c r="C52">
+        <v>455</v>
+      </c>
+      <c r="D52" s="14">
+        <f>C52/B52</f>
+        <v>0.44477028347996089</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="3">
+        <v>45928</v>
+      </c>
+      <c r="B53">
+        <v>1132</v>
+      </c>
+      <c r="C53">
+        <v>370</v>
+      </c>
+      <c r="D53" s="14">
+        <f>C53/B53</f>
+        <v>0.32685512367491165</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="3">
+        <v>45935</v>
+      </c>
+      <c r="B54">
+        <v>1208</v>
+      </c>
+      <c r="C54">
+        <v>383</v>
+      </c>
+      <c r="D54" s="14">
+        <f>C54/B54</f>
+        <v>0.31705298013245031</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="3">
+        <v>45942</v>
+      </c>
+      <c r="B55">
+        <v>1210</v>
+      </c>
+      <c r="C55">
+        <v>368</v>
+      </c>
+      <c r="D55" s="14">
+        <f>C55/B55</f>
+        <v>0.30413223140495865</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="3">
+        <v>45949</v>
+      </c>
+      <c r="B56">
+        <v>1200</v>
+      </c>
+      <c r="C56">
+        <v>437</v>
+      </c>
+      <c r="D56" s="14">
+        <f>C56/B56</f>
+        <v>0.36416666666666669</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="3">
+        <v>45956</v>
+      </c>
+      <c r="B57">
+        <v>1237</v>
+      </c>
+      <c r="C57">
+        <v>364</v>
+      </c>
+      <c r="D57" s="14">
+        <f>C57/B57</f>
+        <v>0.29426030719482621</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="3">
+        <v>45963</v>
+      </c>
+      <c r="B58">
+        <v>1301</v>
+      </c>
+      <c r="C58">
+        <v>363</v>
+      </c>
+      <c r="D58" s="14">
+        <f>C58/B58</f>
+        <v>0.27901614142966946</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="3">
+        <v>45970</v>
+      </c>
+      <c r="B59">
+        <v>1369</v>
+      </c>
+      <c r="C59">
+        <v>390</v>
+      </c>
+      <c r="D59" s="14">
+        <f>C59/B59</f>
+        <v>0.28487947406866326</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="3">
+        <v>45977</v>
+      </c>
+      <c r="B60">
+        <v>1434</v>
+      </c>
+      <c r="C60">
+        <v>432</v>
+      </c>
+      <c r="D60" s="14">
+        <f>C60/B60</f>
+        <v>0.30125523012552302</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="3">
+        <v>45984</v>
+      </c>
+      <c r="B61">
+        <v>1439</v>
+      </c>
+      <c r="C61">
+        <v>427</v>
+      </c>
+      <c r="D61" s="14">
+        <f>C61/B61</f>
+        <v>0.29673384294649063</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="3">
+        <v>45991</v>
+      </c>
+      <c r="B62">
+        <v>1341</v>
+      </c>
+      <c r="C62">
+        <v>248</v>
+      </c>
+      <c r="D62" s="14">
+        <f>C62/B62</f>
+        <v>0.18493661446681581</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="3">
+        <v>45998</v>
+      </c>
+      <c r="B63">
+        <v>1305</v>
+      </c>
+      <c r="C63">
+        <v>417</v>
+      </c>
+      <c r="D63" s="14">
+        <f>C63/B63</f>
+        <v>0.31954022988505748</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="3">
+        <v>46005</v>
+      </c>
+      <c r="B64">
+        <v>1369</v>
+      </c>
+      <c r="C64">
+        <v>465</v>
+      </c>
+      <c r="D64" s="14">
+        <f>C64/B64</f>
+        <v>0.33966398831263694</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="3">
+        <v>46012</v>
+      </c>
+      <c r="B65">
+        <v>1324</v>
+      </c>
+      <c r="C65">
+        <v>363</v>
+      </c>
+      <c r="D65" s="14">
+        <f>C65/B65</f>
+        <v>0.27416918429003023</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="3">
+        <v>46019</v>
+      </c>
+      <c r="B66">
+        <v>1277</v>
+      </c>
+      <c r="C66">
+        <v>228</v>
+      </c>
+      <c r="D66" s="14">
+        <f>C66/B66</f>
+        <v>0.17854346123727485</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="3">
+        <v>46026</v>
+      </c>
+      <c r="B67">
+        <v>1224</v>
+      </c>
+      <c r="C67">
+        <v>250</v>
+      </c>
+      <c r="D67" s="14">
+        <f>C67/B67</f>
+        <v>0.20424836601307189</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="3">
+        <v>46033</v>
+      </c>
+      <c r="B68">
+        <v>1195</v>
+      </c>
+      <c r="C68">
+        <v>199</v>
+      </c>
+      <c r="D68" s="14">
+        <f>C68/B68</f>
+        <v>0.16652719665271967</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="3">
+        <v>46040</v>
+      </c>
+      <c r="B69">
+        <v>1123</v>
+      </c>
+      <c r="C69">
+        <v>281</v>
+      </c>
+      <c r="D69" s="14">
+        <f>C69/B69</f>
+        <v>0.25022261798753337</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update Recruiting Percentage Format
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D153B1F-E668-497F-B099-4759BA530ACA}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1B9EBC2-5770-4599-8EAA-01C417EA76B6}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -175,7 +175,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -196,6 +196,7 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3439,14 +3440,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="3" width="32.85546875" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -3460,7 +3461,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:6">
       <c r="A2" s="3">
         <v>45571</v>
       </c>
@@ -3471,11 +3472,12 @@
         <v>476</v>
       </c>
       <c r="D2" s="16">
-        <f t="shared" ref="D2:D33" si="0">C2/B2</f>
-        <v>0.18986836856800957</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <f>C2/B2*100</f>
+        <v>18.986836856800956</v>
+      </c>
+      <c r="F2" s="18"/>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="3">
         <v>45578</v>
       </c>
@@ -3486,11 +3488,11 @@
         <v>445</v>
       </c>
       <c r="D3" s="16">
-        <f t="shared" si="0"/>
-        <v>0.17907444668008049</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <f t="shared" ref="D3:D66" si="0">C3/B3*100</f>
+        <v>17.907444668008051</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" s="3">
         <v>45585</v>
       </c>
@@ -3502,10 +3504,10 @@
       </c>
       <c r="D4" s="16">
         <f t="shared" si="0"/>
-        <v>0.20157938487115545</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>20.157938487115544</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" s="3">
         <v>45592</v>
       </c>
@@ -3517,10 +3519,10 @@
       </c>
       <c r="D5" s="16">
         <f t="shared" si="0"/>
-        <v>0.23645546372819101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>23.645546372819101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" s="3">
         <v>45599</v>
       </c>
@@ -3532,10 +3534,10 @@
       </c>
       <c r="D6" s="16">
         <f t="shared" si="0"/>
-        <v>0.24939584340260995</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+        <v>24.939584340260996</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" s="3">
         <v>45606</v>
       </c>
@@ -3547,10 +3549,10 @@
       </c>
       <c r="D7" s="16">
         <f t="shared" si="0"/>
-        <v>0.25074775672981059</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+        <v>25.074775672981058</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" s="3">
         <v>45613</v>
       </c>
@@ -3562,10 +3564,10 @@
       </c>
       <c r="D8" s="16">
         <f t="shared" si="0"/>
-        <v>0.23226135783563043</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
+        <v>23.226135783563041</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" s="3">
         <v>45620</v>
       </c>
@@ -3577,10 +3579,10 @@
       </c>
       <c r="D9" s="16">
         <f t="shared" si="0"/>
-        <v>0.37710970464135019</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
+        <v>37.710970464135016</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" s="3">
         <v>45627</v>
       </c>
@@ -3592,10 +3594,10 @@
       </c>
       <c r="D10" s="16">
         <f t="shared" si="0"/>
-        <v>0.18238993710691823</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
+        <v>18.238993710691823</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" s="3">
         <v>45634</v>
       </c>
@@ -3607,10 +3609,10 @@
       </c>
       <c r="D11" s="16">
         <f t="shared" si="0"/>
-        <v>0.35982580293957539</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
+        <v>35.98258029395754</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" s="3">
         <v>45641</v>
       </c>
@@ -3622,10 +3624,10 @@
       </c>
       <c r="D12" s="16">
         <f t="shared" si="0"/>
-        <v>0.31486715658564163</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
+        <v>31.486715658564162</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" s="3">
         <v>45648</v>
       </c>
@@ -3637,10 +3639,10 @@
       </c>
       <c r="D13" s="16">
         <f t="shared" si="0"/>
-        <v>0.22686567164179106</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
+        <v>22.686567164179106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="3">
         <v>45655</v>
       </c>
@@ -3652,10 +3654,10 @@
       </c>
       <c r="D14" s="16">
         <f t="shared" si="0"/>
-        <v>0.13207547169811321</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
+        <v>13.20754716981132</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" s="3">
         <v>45662</v>
       </c>
@@ -3667,10 +3669,10 @@
       </c>
       <c r="D15" s="16">
         <f t="shared" si="0"/>
-        <v>0.17861715749039692</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
+        <v>17.861715749039693</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" s="3">
         <v>45669</v>
       </c>
@@ -3682,7 +3684,7 @@
       </c>
       <c r="D16" s="16">
         <f t="shared" si="0"/>
-        <v>0.17501626545217958</v>
+        <v>17.501626545217956</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -3697,7 +3699,7 @@
       </c>
       <c r="D17" s="16">
         <f t="shared" si="0"/>
-        <v>0.17650876054510059</v>
+        <v>17.650876054510061</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -3712,7 +3714,7 @@
       </c>
       <c r="D18" s="16">
         <f t="shared" si="0"/>
-        <v>0.21300597213005973</v>
+        <v>21.300597213005972</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -3727,7 +3729,7 @@
       </c>
       <c r="D19" s="16">
         <f t="shared" si="0"/>
-        <v>0.28982456140350876</v>
+        <v>28.982456140350877</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -3742,7 +3744,7 @@
       </c>
       <c r="D20" s="16">
         <f t="shared" si="0"/>
-        <v>0.17522871217452499</v>
+        <v>17.522871217452497</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -3757,7 +3759,7 @@
       </c>
       <c r="D21" s="16">
         <f t="shared" si="0"/>
-        <v>0.23297213622291021</v>
+        <v>23.297213622291022</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -3772,7 +3774,7 @@
       </c>
       <c r="D22" s="16">
         <f t="shared" si="0"/>
-        <v>0.22615384615384615</v>
+        <v>22.615384615384613</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -3787,7 +3789,7 @@
       </c>
       <c r="D23" s="16">
         <f t="shared" si="0"/>
-        <v>0.27142857142857141</v>
+        <v>27.142857142857142</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -3802,7 +3804,7 @@
       </c>
       <c r="D24" s="16">
         <f t="shared" si="0"/>
-        <v>0.2656364974245769</v>
+        <v>26.563649742457692</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -3817,7 +3819,7 @@
       </c>
       <c r="D25" s="16">
         <f t="shared" si="0"/>
-        <v>0.21816827997021593</v>
+        <v>21.816827997021594</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -3832,7 +3834,7 @@
       </c>
       <c r="D26" s="16">
         <f t="shared" si="0"/>
-        <v>0.27439024390243905</v>
+        <v>27.439024390243905</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -3847,7 +3849,7 @@
       </c>
       <c r="D27" s="16">
         <f t="shared" si="0"/>
-        <v>0.23930982745686422</v>
+        <v>23.930982745686421</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -3862,7 +3864,7 @@
       </c>
       <c r="D28" s="16">
         <f t="shared" si="0"/>
-        <v>0.27200000000000002</v>
+        <v>27.200000000000003</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -3877,7 +3879,7 @@
       </c>
       <c r="D29" s="16">
         <f t="shared" si="0"/>
-        <v>0.25387755102040815</v>
+        <v>25.387755102040817</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -3892,7 +3894,7 @@
       </c>
       <c r="D30" s="16">
         <f t="shared" si="0"/>
-        <v>0.23102866779089376</v>
+        <v>23.102866779089375</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -3907,7 +3909,7 @@
       </c>
       <c r="D31" s="16">
         <f t="shared" si="0"/>
-        <v>0.35034602076124566</v>
+        <v>35.034602076124564</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -3922,7 +3924,7 @@
       </c>
       <c r="D32" s="16">
         <f t="shared" si="0"/>
-        <v>0.33018056749785041</v>
+        <v>33.018056749785039</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -3937,7 +3939,7 @@
       </c>
       <c r="D33" s="16">
         <f t="shared" si="0"/>
-        <v>0.33187772925764192</v>
+        <v>33.187772925764193</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -3951,8 +3953,8 @@
         <v>363</v>
       </c>
       <c r="D34" s="16">
-        <f t="shared" ref="D34:D65" si="1">C34/B34</f>
-        <v>0.31703056768558951</v>
+        <f t="shared" si="0"/>
+        <v>31.703056768558952</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -3966,8 +3968,8 @@
         <v>342</v>
       </c>
       <c r="D35" s="16">
-        <f t="shared" si="1"/>
-        <v>0.30158730158730157</v>
+        <f t="shared" si="0"/>
+        <v>30.158730158730158</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -3981,8 +3983,8 @@
         <v>293</v>
       </c>
       <c r="D36" s="16">
-        <f t="shared" si="1"/>
-        <v>0.26207513416815742</v>
+        <f t="shared" si="0"/>
+        <v>26.207513416815743</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -3996,8 +3998,8 @@
         <v>375</v>
       </c>
       <c r="D37" s="16">
-        <f t="shared" si="1"/>
-        <v>0.33632286995515698</v>
+        <f t="shared" si="0"/>
+        <v>33.632286995515699</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -4011,8 +4013,8 @@
         <v>288</v>
       </c>
       <c r="D38" s="16">
-        <f t="shared" si="1"/>
-        <v>0.25486725663716814</v>
+        <f t="shared" si="0"/>
+        <v>25.486725663716815</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -4026,8 +4028,8 @@
         <v>257</v>
       </c>
       <c r="D39" s="16">
-        <f t="shared" si="1"/>
-        <v>0.232579185520362</v>
+        <f t="shared" si="0"/>
+        <v>23.257918552036198</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -4041,8 +4043,8 @@
         <v>273</v>
       </c>
       <c r="D40" s="16">
-        <f t="shared" si="1"/>
-        <v>0.24309884238646481</v>
+        <f t="shared" si="0"/>
+        <v>24.309884238646482</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -4056,8 +4058,8 @@
         <v>198</v>
       </c>
       <c r="D41" s="16">
-        <f t="shared" si="1"/>
-        <v>0.18049225159525981</v>
+        <f t="shared" si="0"/>
+        <v>18.049225159525982</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -4071,8 +4073,8 @@
         <v>216</v>
       </c>
       <c r="D42" s="16">
-        <f t="shared" si="1"/>
-        <v>0.20338983050847459</v>
+        <f t="shared" si="0"/>
+        <v>20.33898305084746</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -4086,8 +4088,8 @@
         <v>247</v>
       </c>
       <c r="D43" s="16">
-        <f t="shared" si="1"/>
-        <v>0.23591212989493793</v>
+        <f t="shared" si="0"/>
+        <v>23.591212989493794</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -4101,8 +4103,8 @@
         <v>215</v>
       </c>
       <c r="D44" s="16">
-        <f t="shared" si="1"/>
-        <v>0.21182266009852216</v>
+        <f t="shared" si="0"/>
+        <v>21.182266009852217</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -4116,8 +4118,8 @@
         <v>214</v>
       </c>
       <c r="D45" s="16">
-        <f t="shared" si="1"/>
-        <v>0.21792260692464357</v>
+        <f t="shared" si="0"/>
+        <v>21.792260692464357</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -4131,8 +4133,8 @@
         <v>356</v>
       </c>
       <c r="D46" s="16">
-        <f t="shared" si="1"/>
-        <v>0.36891191709844562</v>
+        <f t="shared" si="0"/>
+        <v>36.891191709844563</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -4146,8 +4148,8 @@
         <v>387</v>
       </c>
       <c r="D47" s="16">
-        <f t="shared" si="1"/>
-        <v>0.40396659707724425</v>
+        <f t="shared" si="0"/>
+        <v>40.396659707724424</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -4161,8 +4163,8 @@
         <v>284</v>
       </c>
       <c r="D48" s="16">
-        <f t="shared" si="1"/>
-        <v>0.27466150870406192</v>
+        <f t="shared" si="0"/>
+        <v>27.466150870406192</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -4176,8 +4178,8 @@
         <v>274</v>
       </c>
       <c r="D49" s="16">
-        <f t="shared" si="1"/>
-        <v>0.26731707317073172</v>
+        <f t="shared" si="0"/>
+        <v>26.731707317073173</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -4191,8 +4193,8 @@
         <v>365</v>
       </c>
       <c r="D50" s="16">
-        <f t="shared" si="1"/>
-        <v>0.3574926542605289</v>
+        <f t="shared" si="0"/>
+        <v>35.749265426052887</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -4206,8 +4208,8 @@
         <v>380</v>
       </c>
       <c r="D51" s="16">
-        <f t="shared" si="1"/>
-        <v>0.37848605577689243</v>
+        <f t="shared" si="0"/>
+        <v>37.848605577689241</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -4221,8 +4223,8 @@
         <v>455</v>
       </c>
       <c r="D52" s="16">
-        <f t="shared" si="1"/>
-        <v>0.44477028347996089</v>
+        <f t="shared" si="0"/>
+        <v>44.47702834799609</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -4236,8 +4238,8 @@
         <v>370</v>
       </c>
       <c r="D53" s="16">
-        <f t="shared" si="1"/>
-        <v>0.32685512367491165</v>
+        <f t="shared" si="0"/>
+        <v>32.685512367491164</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -4251,8 +4253,8 @@
         <v>383</v>
       </c>
       <c r="D54" s="16">
-        <f t="shared" si="1"/>
-        <v>0.31705298013245031</v>
+        <f t="shared" si="0"/>
+        <v>31.705298013245031</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -4266,8 +4268,8 @@
         <v>368</v>
       </c>
       <c r="D55" s="16">
-        <f t="shared" si="1"/>
-        <v>0.30413223140495865</v>
+        <f t="shared" si="0"/>
+        <v>30.413223140495866</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -4281,8 +4283,8 @@
         <v>437</v>
       </c>
       <c r="D56" s="16">
-        <f t="shared" si="1"/>
-        <v>0.36416666666666669</v>
+        <f t="shared" si="0"/>
+        <v>36.416666666666671</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -4296,8 +4298,8 @@
         <v>364</v>
       </c>
       <c r="D57" s="16">
-        <f t="shared" si="1"/>
-        <v>0.29426030719482621</v>
+        <f t="shared" si="0"/>
+        <v>29.426030719482622</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -4311,8 +4313,8 @@
         <v>363</v>
       </c>
       <c r="D58" s="16">
-        <f t="shared" si="1"/>
-        <v>0.27901614142966946</v>
+        <f t="shared" si="0"/>
+        <v>27.901614142966945</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -4326,8 +4328,8 @@
         <v>390</v>
       </c>
       <c r="D59" s="16">
-        <f t="shared" si="1"/>
-        <v>0.28487947406866326</v>
+        <f t="shared" si="0"/>
+        <v>28.487947406866326</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -4341,8 +4343,8 @@
         <v>432</v>
       </c>
       <c r="D60" s="16">
-        <f t="shared" si="1"/>
-        <v>0.30125523012552302</v>
+        <f t="shared" si="0"/>
+        <v>30.125523012552303</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -4356,8 +4358,8 @@
         <v>427</v>
       </c>
       <c r="D61" s="16">
-        <f t="shared" si="1"/>
-        <v>0.29673384294649063</v>
+        <f t="shared" si="0"/>
+        <v>29.673384294649065</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -4371,8 +4373,8 @@
         <v>248</v>
       </c>
       <c r="D62" s="16">
-        <f t="shared" si="1"/>
-        <v>0.18493661446681581</v>
+        <f t="shared" si="0"/>
+        <v>18.493661446681582</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -4386,8 +4388,8 @@
         <v>417</v>
       </c>
       <c r="D63" s="16">
-        <f t="shared" si="1"/>
-        <v>0.31954022988505748</v>
+        <f t="shared" si="0"/>
+        <v>31.954022988505749</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -4401,8 +4403,8 @@
         <v>465</v>
       </c>
       <c r="D64" s="16">
-        <f t="shared" si="1"/>
-        <v>0.33966398831263694</v>
+        <f t="shared" si="0"/>
+        <v>33.966398831263696</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -4416,8 +4418,8 @@
         <v>363</v>
       </c>
       <c r="D65" s="16">
-        <f t="shared" si="1"/>
-        <v>0.27416918429003023</v>
+        <f t="shared" si="0"/>
+        <v>27.416918429003022</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -4431,8 +4433,8 @@
         <v>228</v>
       </c>
       <c r="D66" s="16">
-        <f t="shared" ref="D66:D69" si="2">C66/B66</f>
-        <v>0.17854346123727485</v>
+        <f t="shared" si="0"/>
+        <v>17.854346123727485</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -4446,8 +4448,8 @@
         <v>250</v>
       </c>
       <c r="D67" s="16">
-        <f t="shared" si="2"/>
-        <v>0.20424836601307189</v>
+        <f t="shared" ref="D67:D69" si="1">C67/B67*100</f>
+        <v>20.424836601307188</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -4461,8 +4463,8 @@
         <v>199</v>
       </c>
       <c r="D68" s="16">
-        <f t="shared" si="2"/>
-        <v>0.16652719665271967</v>
+        <f t="shared" si="1"/>
+        <v>16.652719665271967</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -4476,8 +4478,8 @@
         <v>281</v>
       </c>
       <c r="D69" s="16">
-        <f t="shared" si="2"/>
-        <v>0.25022261798753337</v>
+        <f t="shared" si="1"/>
+        <v>25.022261798753338</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data Update WE 1-18-26
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="115" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1B9EBC2-5770-4599-8EAA-01C417EA76B6}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CA9F53A-0B19-48C6-B889-242A73BB3739}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -175,7 +175,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -197,6 +197,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1623,151 +1624,244 @@
       <c r="A56" s="3">
         <v>46040</v>
       </c>
+      <c r="B56" s="6">
+        <v>214041.85999999952</v>
+      </c>
       <c r="C56" s="13">
         <v>278804.31999999972</v>
+      </c>
+      <c r="D56" s="6">
+        <v>20004.82</v>
+      </c>
+      <c r="E56" s="19">
+        <v>0.10290000000000001</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="3">
         <v>46047</v>
       </c>
+      <c r="B57" s="6"/>
       <c r="C57" s="13">
         <v>325526.04999999946</v>
       </c>
+      <c r="D57" s="6"/>
+      <c r="E57" s="19"/>
     </row>
     <row r="58" spans="1:6">
-      <c r="A58" s="3"/>
-      <c r="C58" s="13"/>
+      <c r="A58" s="3">
+        <v>46054</v>
+      </c>
+      <c r="B58" s="6"/>
+      <c r="C58" s="13">
+        <v>310656.64999999967</v>
+      </c>
+      <c r="D58" s="6"/>
+      <c r="E58" s="19"/>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="3"/>
+      <c r="B59" s="6"/>
       <c r="C59" s="13"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="19"/>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="3"/>
+      <c r="B60" s="6"/>
       <c r="C60" s="13"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="19"/>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="3"/>
+      <c r="B61" s="6"/>
       <c r="C61" s="13"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="19"/>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="3"/>
+      <c r="B62" s="6"/>
       <c r="C62" s="13"/>
+      <c r="D62" s="6"/>
+      <c r="E62" s="19"/>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="3"/>
+      <c r="B63" s="6"/>
       <c r="C63" s="13"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="19"/>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="3"/>
+      <c r="B64" s="6"/>
       <c r="C64" s="13"/>
-    </row>
-    <row r="65" spans="1:3">
+      <c r="D64" s="6"/>
+      <c r="E64" s="19"/>
+    </row>
+    <row r="65" spans="1:5">
       <c r="A65" s="3"/>
+      <c r="B65" s="6"/>
       <c r="C65" s="13"/>
-    </row>
-    <row r="66" spans="1:3">
+      <c r="D65" s="6"/>
+      <c r="E65" s="19"/>
+    </row>
+    <row r="66" spans="1:5">
       <c r="A66" s="3"/>
+      <c r="B66" s="6"/>
       <c r="C66" s="13"/>
-    </row>
-    <row r="67" spans="1:3">
+      <c r="D66" s="6"/>
+      <c r="E66" s="19"/>
+    </row>
+    <row r="67" spans="1:5">
       <c r="A67" s="3"/>
+      <c r="B67" s="6"/>
       <c r="C67" s="13"/>
-    </row>
-    <row r="68" spans="1:3">
+      <c r="D67" s="6"/>
+      <c r="E67" s="19"/>
+    </row>
+    <row r="68" spans="1:5">
       <c r="A68" s="3"/>
+      <c r="B68" s="6"/>
       <c r="C68" s="13"/>
-    </row>
-    <row r="69" spans="1:3">
+      <c r="D68" s="6"/>
+      <c r="E68" s="19"/>
+    </row>
+    <row r="69" spans="1:5">
       <c r="A69" s="3"/>
+      <c r="B69" s="6"/>
       <c r="C69" s="13"/>
-    </row>
-    <row r="70" spans="1:3">
+      <c r="D69" s="6"/>
+      <c r="E69" s="19"/>
+    </row>
+    <row r="70" spans="1:5">
       <c r="A70" s="3"/>
+      <c r="B70" s="6"/>
       <c r="C70" s="13"/>
-    </row>
-    <row r="71" spans="1:3">
+      <c r="D70" s="6"/>
+      <c r="E70" s="19"/>
+    </row>
+    <row r="71" spans="1:5">
       <c r="A71" s="3"/>
+      <c r="B71" s="6"/>
       <c r="C71" s="13"/>
-    </row>
-    <row r="72" spans="1:3">
+      <c r="D71" s="6"/>
+      <c r="E71" s="19"/>
+    </row>
+    <row r="72" spans="1:5">
       <c r="A72" s="3"/>
+      <c r="B72" s="6"/>
       <c r="C72" s="13"/>
-    </row>
-    <row r="73" spans="1:3">
+      <c r="D72" s="6"/>
+      <c r="E72" s="19"/>
+    </row>
+    <row r="73" spans="1:5">
       <c r="A73" s="3"/>
+      <c r="B73" s="6"/>
       <c r="C73" s="13"/>
-    </row>
-    <row r="74" spans="1:3">
+      <c r="D73" s="6"/>
+      <c r="E73" s="19"/>
+    </row>
+    <row r="74" spans="1:5">
       <c r="A74" s="3"/>
+      <c r="B74" s="6"/>
       <c r="C74" s="13"/>
-    </row>
-    <row r="75" spans="1:3">
+      <c r="D74" s="6"/>
+      <c r="E74" s="19"/>
+    </row>
+    <row r="75" spans="1:5">
       <c r="A75" s="3"/>
+      <c r="B75" s="6"/>
       <c r="C75" s="13"/>
-    </row>
-    <row r="76" spans="1:3">
+      <c r="D75" s="6"/>
+      <c r="E75" s="19"/>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="B76" s="6"/>
       <c r="C76" s="13"/>
-    </row>
-    <row r="77" spans="1:3">
+      <c r="D76" s="6"/>
+      <c r="E76" s="19"/>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="B77" s="6"/>
       <c r="C77" s="13"/>
-    </row>
-    <row r="78" spans="1:3">
+      <c r="D77" s="6"/>
+      <c r="E77" s="19"/>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="B78" s="6"/>
       <c r="C78" s="13"/>
-    </row>
-    <row r="79" spans="1:3">
+      <c r="D78" s="6"/>
+      <c r="E78" s="19"/>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="B79" s="6"/>
       <c r="C79" s="13"/>
-    </row>
-    <row r="80" spans="1:3">
+      <c r="D79" s="6"/>
+      <c r="E79" s="19"/>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="B80" s="6"/>
       <c r="C80" s="13"/>
-    </row>
-    <row r="81" spans="3:3">
+      <c r="D80" s="6"/>
+      <c r="E80" s="19"/>
+    </row>
+    <row r="81" spans="3:5">
       <c r="C81" s="13"/>
-    </row>
-    <row r="82" spans="3:3">
+      <c r="E81" s="19"/>
+    </row>
+    <row r="82" spans="3:5">
       <c r="C82" s="13"/>
-    </row>
-    <row r="83" spans="3:3">
+      <c r="E82" s="19"/>
+    </row>
+    <row r="83" spans="3:5">
       <c r="C83" s="13"/>
-    </row>
-    <row r="84" spans="3:3">
+      <c r="E83" s="19"/>
+    </row>
+    <row r="84" spans="3:5">
       <c r="C84" s="13"/>
-    </row>
-    <row r="85" spans="3:3">
+      <c r="E84" s="19"/>
+    </row>
+    <row r="85" spans="3:5">
       <c r="C85" s="13"/>
-    </row>
-    <row r="86" spans="3:3">
+      <c r="E85" s="19"/>
+    </row>
+    <row r="86" spans="3:5">
       <c r="C86" s="13"/>
-    </row>
-    <row r="87" spans="3:3">
+      <c r="E86" s="19"/>
+    </row>
+    <row r="87" spans="3:5">
       <c r="C87" s="13"/>
-    </row>
-    <row r="88" spans="3:3">
+      <c r="E87" s="19"/>
+    </row>
+    <row r="88" spans="3:5">
       <c r="C88" s="13"/>
-    </row>
-    <row r="89" spans="3:3">
+      <c r="E88" s="19"/>
+    </row>
+    <row r="89" spans="3:5">
       <c r="C89" s="13"/>
     </row>
-    <row r="90" spans="3:3">
+    <row r="90" spans="3:5">
       <c r="C90" s="13"/>
     </row>
-    <row r="91" spans="3:3">
+    <row r="91" spans="3:5">
       <c r="C91" s="13"/>
     </row>
-    <row r="92" spans="3:3">
+    <row r="92" spans="3:5">
       <c r="C92" s="13"/>
     </row>
-    <row r="93" spans="3:3">
+    <row r="93" spans="3:5">
       <c r="C93" s="13"/>
     </row>
-    <row r="94" spans="3:3">
+    <row r="94" spans="3:5">
       <c r="C94" s="13"/>
     </row>
-    <row r="95" spans="3:3">
+    <row r="95" spans="3:5">
       <c r="C95" s="13"/>
     </row>
-    <row r="96" spans="3:3">
+    <row r="96" spans="3:5">
       <c r="C96" s="13"/>
     </row>
     <row r="97" spans="3:3">
@@ -2920,11 +3014,17 @@
       <c r="B56">
         <v>733</v>
       </c>
+      <c r="C56">
+        <v>802</v>
+      </c>
       <c r="E56" s="3">
         <v>46040</v>
       </c>
       <c r="F56">
         <v>0.97989999999999999</v>
+      </c>
+      <c r="G56">
+        <v>0.98160000000000003</v>
       </c>
     </row>
     <row r="57" spans="1:7">

</xml_diff>

<commit_message>
Week ending 1-25-26 data update
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="132" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CA9F53A-0B19-48C6-B889-242A73BB3739}"/>
+  <xr:revisionPtr revIDLastSave="157" documentId="8_{AE5846BF-940B-4D2C-884D-E857B5928A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BDADBB3-094B-43A0-9FC1-D5C2F48F4033}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1641,12 +1641,18 @@
       <c r="A57" s="3">
         <v>46047</v>
       </c>
-      <c r="B57" s="6"/>
+      <c r="B57" s="6">
+        <v>211496.52000000025</v>
+      </c>
       <c r="C57" s="13">
         <v>325526.04999999946</v>
       </c>
-      <c r="D57" s="6"/>
-      <c r="E57" s="19"/>
+      <c r="D57" s="6">
+        <v>17217.009999999998</v>
+      </c>
+      <c r="E57" s="19">
+        <v>8.1405642040824025E-2</v>
+      </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="3">
@@ -3034,11 +3040,17 @@
       <c r="B57">
         <v>845</v>
       </c>
+      <c r="C57">
+        <v>780</v>
+      </c>
       <c r="E57" s="3">
         <v>46047</v>
       </c>
       <c r="F57">
         <v>0.98</v>
+      </c>
+      <c r="G57">
+        <v>0.96179999999999999</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -3540,7 +3552,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="3" width="32.85546875" customWidth="1"/>
@@ -4548,7 +4560,7 @@
         <v>250</v>
       </c>
       <c r="D67" s="16">
-        <f t="shared" ref="D67:D69" si="1">C67/B67*100</f>
+        <f t="shared" ref="D67:D70" si="1">C67/B67*100</f>
         <v>20.424836601307188</v>
       </c>
     </row>
@@ -4580,6 +4592,21 @@
       <c r="D69" s="16">
         <f t="shared" si="1"/>
         <v>25.022261798753338</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="3">
+        <v>46047</v>
+      </c>
+      <c r="B70">
+        <v>1060</v>
+      </c>
+      <c r="C70">
+        <v>315</v>
+      </c>
+      <c r="D70" s="17">
+        <f t="shared" si="1"/>
+        <v>29.716981132075471</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data Update WE 2-1-26
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CA5D4CC-235F-4E08-84BA-FA2B7AE289BD}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A85E5B85-6F50-450F-AA55-7025F2ED9F35}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1658,12 +1658,18 @@
       <c r="A58" s="3">
         <v>46054</v>
       </c>
-      <c r="B58" s="6"/>
+      <c r="B58" s="6">
+        <v>185148.03</v>
+      </c>
       <c r="C58" s="13">
         <v>310656.64999999967</v>
       </c>
-      <c r="D58" s="6"/>
-      <c r="E58" s="19"/>
+      <c r="D58" s="6">
+        <v>17748.599999999999</v>
+      </c>
+      <c r="E58" s="19">
+        <v>9.5861673494446575E-2</v>
+      </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="3"/>
@@ -3060,11 +3066,17 @@
       <c r="B58">
         <v>1038</v>
       </c>
+      <c r="C58">
+        <v>708</v>
+      </c>
       <c r="E58" s="3">
         <v>46054</v>
       </c>
       <c r="F58">
         <v>0.97460000000000002</v>
+      </c>
+      <c r="G58">
+        <v>0.9607</v>
       </c>
     </row>
     <row r="59" spans="1:7">
@@ -3547,7 +3559,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="3" width="32.85546875" customWidth="1"/>
@@ -4603,6 +4615,20 @@
         <v>29.72</v>
       </c>
     </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="3">
+        <v>46054</v>
+      </c>
+      <c r="B71">
+        <v>1057</v>
+      </c>
+      <c r="C71">
+        <v>276</v>
+      </c>
+      <c r="D71" s="17">
+        <v>26.11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Adding Ad Clicks and Clickboarding Data
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A85E5B85-6F50-450F-AA55-7025F2ED9F35}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EDC60E5-7D76-4A89-AE29-EA567665964C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>2025 Revenue</t>
   </si>
@@ -86,6 +86,12 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>Ad Clicks</t>
+  </si>
+  <si>
+    <t>Clickboarding Applicants</t>
   </si>
 </sst>
 </file>
@@ -175,7 +181,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -196,7 +202,6 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -1633,7 +1638,7 @@
       <c r="D56" s="6">
         <v>20004.82</v>
       </c>
-      <c r="E56" s="19">
+      <c r="E56" s="18">
         <v>0.10290000000000001</v>
       </c>
     </row>
@@ -1650,7 +1655,7 @@
       <c r="D57" s="6">
         <v>17217.009999999998</v>
       </c>
-      <c r="E57" s="19">
+      <c r="E57" s="18">
         <v>8.1405642040824122E-2</v>
       </c>
     </row>
@@ -1667,7 +1672,7 @@
       <c r="D58" s="6">
         <v>17748.599999999999</v>
       </c>
-      <c r="E58" s="19">
+      <c r="E58" s="18">
         <v>9.5861673494446575E-2</v>
       </c>
     </row>
@@ -1676,181 +1681,181 @@
       <c r="B59" s="6"/>
       <c r="C59" s="13"/>
       <c r="D59" s="6"/>
-      <c r="E59" s="19"/>
+      <c r="E59" s="18"/>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="3"/>
       <c r="B60" s="6"/>
       <c r="C60" s="13"/>
       <c r="D60" s="6"/>
-      <c r="E60" s="19"/>
+      <c r="E60" s="18"/>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="3"/>
       <c r="B61" s="6"/>
       <c r="C61" s="13"/>
       <c r="D61" s="6"/>
-      <c r="E61" s="19"/>
+      <c r="E61" s="18"/>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="3"/>
       <c r="B62" s="6"/>
       <c r="C62" s="13"/>
       <c r="D62" s="6"/>
-      <c r="E62" s="19"/>
+      <c r="E62" s="18"/>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="3"/>
       <c r="B63" s="6"/>
       <c r="C63" s="13"/>
       <c r="D63" s="6"/>
-      <c r="E63" s="19"/>
+      <c r="E63" s="18"/>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="3"/>
       <c r="B64" s="6"/>
       <c r="C64" s="13"/>
       <c r="D64" s="6"/>
-      <c r="E64" s="19"/>
+      <c r="E64" s="18"/>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="3"/>
       <c r="B65" s="6"/>
       <c r="C65" s="13"/>
       <c r="D65" s="6"/>
-      <c r="E65" s="19"/>
+      <c r="E65" s="18"/>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" s="3"/>
       <c r="B66" s="6"/>
       <c r="C66" s="13"/>
       <c r="D66" s="6"/>
-      <c r="E66" s="19"/>
+      <c r="E66" s="18"/>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="3"/>
       <c r="B67" s="6"/>
       <c r="C67" s="13"/>
       <c r="D67" s="6"/>
-      <c r="E67" s="19"/>
+      <c r="E67" s="18"/>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" s="3"/>
       <c r="B68" s="6"/>
       <c r="C68" s="13"/>
       <c r="D68" s="6"/>
-      <c r="E68" s="19"/>
+      <c r="E68" s="18"/>
     </row>
     <row r="69" spans="1:5">
       <c r="A69" s="3"/>
       <c r="B69" s="6"/>
       <c r="C69" s="13"/>
       <c r="D69" s="6"/>
-      <c r="E69" s="19"/>
+      <c r="E69" s="18"/>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" s="3"/>
       <c r="B70" s="6"/>
       <c r="C70" s="13"/>
       <c r="D70" s="6"/>
-      <c r="E70" s="19"/>
+      <c r="E70" s="18"/>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="3"/>
       <c r="B71" s="6"/>
       <c r="C71" s="13"/>
       <c r="D71" s="6"/>
-      <c r="E71" s="19"/>
+      <c r="E71" s="18"/>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="3"/>
       <c r="B72" s="6"/>
       <c r="C72" s="13"/>
       <c r="D72" s="6"/>
-      <c r="E72" s="19"/>
+      <c r="E72" s="18"/>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" s="3"/>
       <c r="B73" s="6"/>
       <c r="C73" s="13"/>
       <c r="D73" s="6"/>
-      <c r="E73" s="19"/>
+      <c r="E73" s="18"/>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" s="3"/>
       <c r="B74" s="6"/>
       <c r="C74" s="13"/>
       <c r="D74" s="6"/>
-      <c r="E74" s="19"/>
+      <c r="E74" s="18"/>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" s="3"/>
       <c r="B75" s="6"/>
       <c r="C75" s="13"/>
       <c r="D75" s="6"/>
-      <c r="E75" s="19"/>
+      <c r="E75" s="18"/>
     </row>
     <row r="76" spans="1:5">
       <c r="B76" s="6"/>
       <c r="C76" s="13"/>
       <c r="D76" s="6"/>
-      <c r="E76" s="19"/>
+      <c r="E76" s="18"/>
     </row>
     <row r="77" spans="1:5">
       <c r="B77" s="6"/>
       <c r="C77" s="13"/>
       <c r="D77" s="6"/>
-      <c r="E77" s="19"/>
+      <c r="E77" s="18"/>
     </row>
     <row r="78" spans="1:5">
       <c r="B78" s="6"/>
       <c r="C78" s="13"/>
       <c r="D78" s="6"/>
-      <c r="E78" s="19"/>
+      <c r="E78" s="18"/>
     </row>
     <row r="79" spans="1:5">
       <c r="B79" s="6"/>
       <c r="C79" s="13"/>
       <c r="D79" s="6"/>
-      <c r="E79" s="19"/>
+      <c r="E79" s="18"/>
     </row>
     <row r="80" spans="1:5">
       <c r="B80" s="6"/>
       <c r="C80" s="13"/>
       <c r="D80" s="6"/>
-      <c r="E80" s="19"/>
+      <c r="E80" s="18"/>
     </row>
     <row r="81" spans="3:5">
       <c r="C81" s="13"/>
-      <c r="E81" s="19"/>
+      <c r="E81" s="18"/>
     </row>
     <row r="82" spans="3:5">
       <c r="C82" s="13"/>
-      <c r="E82" s="19"/>
+      <c r="E82" s="18"/>
     </row>
     <row r="83" spans="3:5">
       <c r="C83" s="13"/>
-      <c r="E83" s="19"/>
+      <c r="E83" s="18"/>
     </row>
     <row r="84" spans="3:5">
       <c r="C84" s="13"/>
-      <c r="E84" s="19"/>
+      <c r="E84" s="18"/>
     </row>
     <row r="85" spans="3:5">
       <c r="C85" s="13"/>
-      <c r="E85" s="19"/>
+      <c r="E85" s="18"/>
     </row>
     <row r="86" spans="3:5">
       <c r="C86" s="13"/>
-      <c r="E86" s="19"/>
+      <c r="E86" s="18"/>
     </row>
     <row r="87" spans="3:5">
       <c r="C87" s="13"/>
-      <c r="E87" s="19"/>
+      <c r="E87" s="18"/>
     </row>
     <row r="88" spans="3:5">
       <c r="C88" s="13"/>
-      <c r="E88" s="19"/>
+      <c r="E88" s="18"/>
     </row>
     <row r="89" spans="3:5">
       <c r="C89" s="13"/>
@@ -3564,6 +3569,8 @@
   <cols>
     <col min="1" max="3" width="32.85546875" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" style="17" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3579,6 +3586,12 @@
       <c r="D1" s="15" t="s">
         <v>14</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3">
@@ -3594,7 +3607,12 @@
         <f>C2/B2*100</f>
         <v>18.986836856800956</v>
       </c>
-      <c r="F2" s="18"/>
+      <c r="E2">
+        <v>1757</v>
+      </c>
+      <c r="F2">
+        <v>392</v>
+      </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3">
@@ -3610,6 +3628,12 @@
         <f t="shared" ref="D3:D66" si="0">C3/B3*100</f>
         <v>17.907444668008051</v>
       </c>
+      <c r="E3">
+        <v>2082</v>
+      </c>
+      <c r="F3">
+        <v>380</v>
+      </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3">
@@ -3625,6 +3649,12 @@
         <f t="shared" si="0"/>
         <v>20.157938487115544</v>
       </c>
+      <c r="E4">
+        <v>1820</v>
+      </c>
+      <c r="F4">
+        <v>303</v>
+      </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3">
@@ -3640,6 +3670,12 @@
         <f t="shared" si="0"/>
         <v>23.645546372819101</v>
       </c>
+      <c r="E5">
+        <v>1249</v>
+      </c>
+      <c r="F5">
+        <v>234</v>
+      </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3">
@@ -3655,6 +3691,12 @@
         <f t="shared" si="0"/>
         <v>24.939584340260996</v>
       </c>
+      <c r="E6">
+        <v>957</v>
+      </c>
+      <c r="F6">
+        <v>244</v>
+      </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3">
@@ -3670,6 +3712,12 @@
         <f t="shared" si="0"/>
         <v>25.074775672981058</v>
       </c>
+      <c r="E7">
+        <v>1695</v>
+      </c>
+      <c r="F7">
+        <v>244</v>
+      </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3">
@@ -3685,6 +3733,12 @@
         <f t="shared" si="0"/>
         <v>23.226135783563041</v>
       </c>
+      <c r="E8">
+        <v>1694</v>
+      </c>
+      <c r="F8">
+        <v>283</v>
+      </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3">
@@ -3700,6 +3754,12 @@
         <f t="shared" si="0"/>
         <v>37.710970464135016</v>
       </c>
+      <c r="E9">
+        <v>865</v>
+      </c>
+      <c r="F9">
+        <v>235</v>
+      </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3">
@@ -3715,6 +3775,12 @@
         <f t="shared" si="0"/>
         <v>18.238993710691823</v>
       </c>
+      <c r="E10">
+        <v>522</v>
+      </c>
+      <c r="F10">
+        <v>156</v>
+      </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="3">
@@ -3730,6 +3796,12 @@
         <f t="shared" si="0"/>
         <v>35.98258029395754</v>
       </c>
+      <c r="E11">
+        <v>695</v>
+      </c>
+      <c r="F11">
+        <v>175</v>
+      </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3">
@@ -3745,6 +3817,12 @@
         <f t="shared" si="0"/>
         <v>31.486715658564162</v>
       </c>
+      <c r="E12">
+        <v>323</v>
+      </c>
+      <c r="F12">
+        <v>102</v>
+      </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="3">
@@ -3760,6 +3838,12 @@
         <f t="shared" si="0"/>
         <v>22.686567164179106</v>
       </c>
+      <c r="E13">
+        <v>762</v>
+      </c>
+      <c r="F13">
+        <v>211</v>
+      </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="3">
@@ -3775,6 +3859,12 @@
         <f t="shared" si="0"/>
         <v>13.20754716981132</v>
       </c>
+      <c r="E14" s="14">
+        <v>1038</v>
+      </c>
+      <c r="F14">
+        <v>231</v>
+      </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="3">
@@ -3790,6 +3880,12 @@
         <f t="shared" si="0"/>
         <v>17.861715749039693</v>
       </c>
+      <c r="E15">
+        <v>991</v>
+      </c>
+      <c r="F15">
+        <v>218</v>
+      </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="3">
@@ -3805,8 +3901,14 @@
         <f t="shared" si="0"/>
         <v>17.501626545217956</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16">
+        <v>1637</v>
+      </c>
+      <c r="F16">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" s="3">
         <v>45676</v>
       </c>
@@ -3820,8 +3922,14 @@
         <f t="shared" si="0"/>
         <v>17.650876054510061</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17">
+        <v>1756</v>
+      </c>
+      <c r="F17">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" s="3">
         <v>45683</v>
       </c>
@@ -3835,8 +3943,14 @@
         <f t="shared" si="0"/>
         <v>21.300597213005972</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="E18">
+        <v>1144</v>
+      </c>
+      <c r="F18">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" s="3">
         <v>45690</v>
       </c>
@@ -3850,8 +3964,14 @@
         <f t="shared" si="0"/>
         <v>28.982456140350877</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="E19">
+        <v>710</v>
+      </c>
+      <c r="F19">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" s="3">
         <v>45697</v>
       </c>
@@ -3865,8 +3985,14 @@
         <f t="shared" si="0"/>
         <v>17.522871217452497</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="E20">
+        <v>1564</v>
+      </c>
+      <c r="F20">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" s="3">
         <v>45704</v>
       </c>
@@ -3880,8 +4006,14 @@
         <f t="shared" si="0"/>
         <v>23.297213622291022</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="E21">
+        <v>1283</v>
+      </c>
+      <c r="F21">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22" s="3">
         <v>45711</v>
       </c>
@@ -3895,8 +4027,14 @@
         <f t="shared" si="0"/>
         <v>22.615384615384613</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="E22">
+        <v>1014</v>
+      </c>
+      <c r="F22">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23" s="3">
         <v>45718</v>
       </c>
@@ -3910,8 +4048,14 @@
         <f t="shared" si="0"/>
         <v>27.142857142857142</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="E23">
+        <v>64</v>
+      </c>
+      <c r="F23">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24" s="3">
         <v>45725</v>
       </c>
@@ -3925,8 +4069,14 @@
         <f t="shared" si="0"/>
         <v>26.563649742457692</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="E24">
+        <v>400</v>
+      </c>
+      <c r="F24">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25" s="3">
         <v>45732</v>
       </c>
@@ -3940,8 +4090,14 @@
         <f t="shared" si="0"/>
         <v>21.816827997021594</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="E25">
+        <v>500</v>
+      </c>
+      <c r="F25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26" s="3">
         <v>45739</v>
       </c>
@@ -3955,8 +4111,14 @@
         <f t="shared" si="0"/>
         <v>27.439024390243905</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="E26">
+        <v>408</v>
+      </c>
+      <c r="F26">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27" s="3">
         <v>45746</v>
       </c>
@@ -3970,8 +4132,14 @@
         <f t="shared" si="0"/>
         <v>23.930982745686421</v>
       </c>
-    </row>
-    <row r="28" spans="1:4">
+      <c r="E27">
+        <v>276</v>
+      </c>
+      <c r="F27">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28" s="3">
         <v>45753</v>
       </c>
@@ -3985,8 +4153,14 @@
         <f t="shared" si="0"/>
         <v>27.200000000000003</v>
       </c>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="E28">
+        <v>385</v>
+      </c>
+      <c r="F28">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29" s="3">
         <v>45760</v>
       </c>
@@ -4000,8 +4174,14 @@
         <f t="shared" si="0"/>
         <v>25.387755102040817</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="E29">
+        <v>575</v>
+      </c>
+      <c r="F29">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30" s="3">
         <v>45767</v>
       </c>
@@ -4015,8 +4195,14 @@
         <f t="shared" si="0"/>
         <v>23.102866779089375</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
+      <c r="E30">
+        <v>406</v>
+      </c>
+      <c r="F30">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
       <c r="A31" s="3">
         <v>45774</v>
       </c>
@@ -4030,8 +4216,14 @@
         <f t="shared" si="0"/>
         <v>35.034602076124564</v>
       </c>
-    </row>
-    <row r="32" spans="1:4">
+      <c r="E31">
+        <v>786</v>
+      </c>
+      <c r="F31">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32" s="3">
         <v>45781</v>
       </c>
@@ -4045,8 +4237,14 @@
         <f t="shared" si="0"/>
         <v>33.018056749785039</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="E32">
+        <v>794</v>
+      </c>
+      <c r="F32">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33" s="3">
         <v>45788</v>
       </c>
@@ -4060,8 +4258,14 @@
         <f t="shared" si="0"/>
         <v>33.187772925764193</v>
       </c>
-    </row>
-    <row r="34" spans="1:4">
+      <c r="E33">
+        <v>923</v>
+      </c>
+      <c r="F33">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34" s="3">
         <v>45795</v>
       </c>
@@ -4075,8 +4279,14 @@
         <f t="shared" si="0"/>
         <v>31.703056768558952</v>
       </c>
-    </row>
-    <row r="35" spans="1:4">
+      <c r="E34">
+        <v>845</v>
+      </c>
+      <c r="F34">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
       <c r="A35" s="3">
         <v>45802</v>
       </c>
@@ -4090,8 +4300,14 @@
         <f t="shared" si="0"/>
         <v>30.158730158730158</v>
       </c>
-    </row>
-    <row r="36" spans="1:4">
+      <c r="E35">
+        <v>675</v>
+      </c>
+      <c r="F35">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36" s="3">
         <v>45809</v>
       </c>
@@ -4105,8 +4321,14 @@
         <f t="shared" si="0"/>
         <v>26.207513416815743</v>
       </c>
-    </row>
-    <row r="37" spans="1:4">
+      <c r="E36">
+        <v>365</v>
+      </c>
+      <c r="F36">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37" s="3">
         <v>45816</v>
       </c>
@@ -4120,8 +4342,14 @@
         <f t="shared" si="0"/>
         <v>33.632286995515699</v>
       </c>
-    </row>
-    <row r="38" spans="1:4">
+      <c r="E37">
+        <v>780</v>
+      </c>
+      <c r="F37">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
       <c r="A38" s="3">
         <v>45823</v>
       </c>
@@ -4135,8 +4363,14 @@
         <f t="shared" si="0"/>
         <v>25.486725663716815</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
+      <c r="E38">
+        <v>687</v>
+      </c>
+      <c r="F38">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
       <c r="A39" s="3">
         <v>45830</v>
       </c>
@@ -4150,8 +4384,14 @@
         <f t="shared" si="0"/>
         <v>23.257918552036198</v>
       </c>
-    </row>
-    <row r="40" spans="1:4">
+      <c r="E39" s="14">
+        <v>610</v>
+      </c>
+      <c r="F39">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
       <c r="A40" s="3">
         <v>45837</v>
       </c>
@@ -4165,8 +4405,14 @@
         <f t="shared" si="0"/>
         <v>24.309884238646482</v>
       </c>
-    </row>
-    <row r="41" spans="1:4">
+      <c r="E40" s="14">
+        <v>480</v>
+      </c>
+      <c r="F40">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
       <c r="A41" s="3">
         <v>45844</v>
       </c>
@@ -4180,8 +4426,14 @@
         <f t="shared" si="0"/>
         <v>18.049225159525982</v>
       </c>
-    </row>
-    <row r="42" spans="1:4">
+      <c r="E41">
+        <v>364</v>
+      </c>
+      <c r="F41">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
       <c r="A42" s="3">
         <v>45851</v>
       </c>
@@ -4195,8 +4447,14 @@
         <f t="shared" si="0"/>
         <v>20.33898305084746</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
+      <c r="E42">
+        <v>598</v>
+      </c>
+      <c r="F42">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
       <c r="A43" s="3">
         <v>45858</v>
       </c>
@@ -4210,8 +4468,14 @@
         <f t="shared" si="0"/>
         <v>23.591212989493794</v>
       </c>
-    </row>
-    <row r="44" spans="1:4">
+      <c r="E43">
+        <v>618</v>
+      </c>
+      <c r="F43">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
       <c r="A44" s="3">
         <v>45865</v>
       </c>
@@ -4225,8 +4489,14 @@
         <f t="shared" si="0"/>
         <v>21.182266009852217</v>
       </c>
-    </row>
-    <row r="45" spans="1:4">
+      <c r="E44">
+        <v>721</v>
+      </c>
+      <c r="F44">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
       <c r="A45" s="3">
         <v>45872</v>
       </c>
@@ -4240,8 +4510,14 @@
         <f t="shared" si="0"/>
         <v>21.792260692464357</v>
       </c>
-    </row>
-    <row r="46" spans="1:4">
+      <c r="E45">
+        <v>659</v>
+      </c>
+      <c r="F45">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
       <c r="A46" s="3">
         <v>45879</v>
       </c>
@@ -4255,8 +4531,14 @@
         <f t="shared" si="0"/>
         <v>36.891191709844563</v>
       </c>
-    </row>
-    <row r="47" spans="1:4">
+      <c r="E46">
+        <v>710</v>
+      </c>
+      <c r="F46">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
       <c r="A47" s="3">
         <v>45886</v>
       </c>
@@ -4270,8 +4552,14 @@
         <f t="shared" si="0"/>
         <v>40.396659707724424</v>
       </c>
-    </row>
-    <row r="48" spans="1:4">
+      <c r="E47">
+        <v>927</v>
+      </c>
+      <c r="F47">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
       <c r="A48" s="3">
         <v>45893</v>
       </c>
@@ -4285,8 +4573,14 @@
         <f t="shared" si="0"/>
         <v>27.466150870406192</v>
       </c>
-    </row>
-    <row r="49" spans="1:4">
+      <c r="E48">
+        <v>492</v>
+      </c>
+      <c r="F48">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
       <c r="A49" s="3">
         <v>45900</v>
       </c>
@@ -4300,8 +4594,14 @@
         <f t="shared" si="0"/>
         <v>26.731707317073173</v>
       </c>
-    </row>
-    <row r="50" spans="1:4">
+      <c r="E49">
+        <v>356</v>
+      </c>
+      <c r="F49">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
       <c r="A50" s="3">
         <v>45907</v>
       </c>
@@ -4315,8 +4615,14 @@
         <f t="shared" si="0"/>
         <v>35.749265426052887</v>
       </c>
-    </row>
-    <row r="51" spans="1:4">
+      <c r="E50">
+        <v>560</v>
+      </c>
+      <c r="F50">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
       <c r="A51" s="3">
         <v>45914</v>
       </c>
@@ -4330,8 +4636,14 @@
         <f t="shared" si="0"/>
         <v>37.848605577689241</v>
       </c>
-    </row>
-    <row r="52" spans="1:4">
+      <c r="E51">
+        <v>1302</v>
+      </c>
+      <c r="F51">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
       <c r="A52" s="3">
         <v>45921</v>
       </c>
@@ -4345,8 +4657,14 @@
         <f t="shared" si="0"/>
         <v>44.47702834799609</v>
       </c>
-    </row>
-    <row r="53" spans="1:4">
+      <c r="E52">
+        <v>1511</v>
+      </c>
+      <c r="F52">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
       <c r="A53" s="3">
         <v>45928</v>
       </c>
@@ -4360,8 +4678,14 @@
         <f t="shared" si="0"/>
         <v>32.685512367491164</v>
       </c>
-    </row>
-    <row r="54" spans="1:4">
+      <c r="E53">
+        <v>559</v>
+      </c>
+      <c r="F53">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
       <c r="A54" s="3">
         <v>45935</v>
       </c>
@@ -4375,8 +4699,14 @@
         <f t="shared" si="0"/>
         <v>31.705298013245031</v>
       </c>
-    </row>
-    <row r="55" spans="1:4">
+      <c r="E54">
+        <v>921</v>
+      </c>
+      <c r="F54">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
       <c r="A55" s="3">
         <v>45942</v>
       </c>
@@ -4390,8 +4720,14 @@
         <f t="shared" si="0"/>
         <v>30.413223140495866</v>
       </c>
-    </row>
-    <row r="56" spans="1:4">
+      <c r="E55">
+        <v>684</v>
+      </c>
+      <c r="F55">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
       <c r="A56" s="3">
         <v>45949</v>
       </c>
@@ -4405,8 +4741,14 @@
         <f t="shared" si="0"/>
         <v>36.416666666666671</v>
       </c>
-    </row>
-    <row r="57" spans="1:4">
+      <c r="E56">
+        <v>728</v>
+      </c>
+      <c r="F56">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
       <c r="A57" s="3">
         <v>45956</v>
       </c>
@@ -4420,8 +4762,14 @@
         <f t="shared" si="0"/>
         <v>29.426030719482622</v>
       </c>
-    </row>
-    <row r="58" spans="1:4">
+      <c r="E57">
+        <v>1501</v>
+      </c>
+      <c r="F57">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
       <c r="A58" s="3">
         <v>45963</v>
       </c>
@@ -4435,8 +4783,14 @@
         <f t="shared" si="0"/>
         <v>27.901614142966945</v>
       </c>
-    </row>
-    <row r="59" spans="1:4">
+      <c r="E58">
+        <v>1023</v>
+      </c>
+      <c r="F58">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
       <c r="A59" s="3">
         <v>45970</v>
       </c>
@@ -4450,8 +4804,14 @@
         <f t="shared" si="0"/>
         <v>28.487947406866326</v>
       </c>
-    </row>
-    <row r="60" spans="1:4">
+      <c r="E59">
+        <v>1322</v>
+      </c>
+      <c r="F59">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
       <c r="A60" s="3">
         <v>45977</v>
       </c>
@@ -4465,8 +4825,14 @@
         <f t="shared" si="0"/>
         <v>30.125523012552303</v>
       </c>
-    </row>
-    <row r="61" spans="1:4">
+      <c r="E60">
+        <v>1654</v>
+      </c>
+      <c r="F60">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
       <c r="A61" s="3">
         <v>45984</v>
       </c>
@@ -4480,8 +4846,14 @@
         <f t="shared" si="0"/>
         <v>29.673384294649065</v>
       </c>
-    </row>
-    <row r="62" spans="1:4">
+      <c r="E61">
+        <v>2181</v>
+      </c>
+      <c r="F61">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
       <c r="A62" s="3">
         <v>45991</v>
       </c>
@@ -4495,8 +4867,14 @@
         <f t="shared" si="0"/>
         <v>18.493661446681582</v>
       </c>
-    </row>
-    <row r="63" spans="1:4">
+      <c r="E62">
+        <v>585</v>
+      </c>
+      <c r="F62">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
       <c r="A63" s="3">
         <v>45998</v>
       </c>
@@ -4510,8 +4888,14 @@
         <f t="shared" si="0"/>
         <v>31.954022988505749</v>
       </c>
-    </row>
-    <row r="64" spans="1:4">
+      <c r="E63">
+        <v>2122</v>
+      </c>
+      <c r="F63">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
       <c r="A64" s="3">
         <v>46005</v>
       </c>
@@ -4525,8 +4909,14 @@
         <f t="shared" si="0"/>
         <v>33.966398831263696</v>
       </c>
-    </row>
-    <row r="65" spans="1:4">
+      <c r="E64">
+        <v>1543</v>
+      </c>
+      <c r="F64">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
       <c r="A65" s="3">
         <v>46012</v>
       </c>
@@ -4540,8 +4930,14 @@
         <f t="shared" si="0"/>
         <v>27.416918429003022</v>
       </c>
-    </row>
-    <row r="66" spans="1:4">
+      <c r="E65">
+        <v>462</v>
+      </c>
+      <c r="F65">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
       <c r="A66" s="3">
         <v>46019</v>
       </c>
@@ -4555,8 +4951,14 @@
         <f t="shared" si="0"/>
         <v>17.854346123727485</v>
       </c>
-    </row>
-    <row r="67" spans="1:4">
+      <c r="E66">
+        <v>2</v>
+      </c>
+      <c r="F66">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
       <c r="A67" s="3">
         <v>46026</v>
       </c>
@@ -4570,8 +4972,14 @@
         <f t="shared" ref="D67:D69" si="1">C67/B67*100</f>
         <v>20.424836601307188</v>
       </c>
-    </row>
-    <row r="68" spans="1:4">
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
       <c r="A68" s="3">
         <v>46033</v>
       </c>
@@ -4585,8 +4993,14 @@
         <f t="shared" si="1"/>
         <v>16.652719665271967</v>
       </c>
-    </row>
-    <row r="69" spans="1:4">
+      <c r="E68">
+        <v>1</v>
+      </c>
+      <c r="F68">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
       <c r="A69" s="3">
         <v>46040</v>
       </c>
@@ -4600,8 +5014,14 @@
         <f t="shared" si="1"/>
         <v>25.022261798753338</v>
       </c>
-    </row>
-    <row r="70" spans="1:4">
+      <c r="E69">
+        <v>89</v>
+      </c>
+      <c r="F69">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
       <c r="A70" s="3">
         <v>46047</v>
       </c>
@@ -4614,8 +5034,14 @@
       <c r="D70" s="17">
         <v>29.72</v>
       </c>
-    </row>
-    <row r="71" spans="1:4">
+      <c r="E70">
+        <v>101</v>
+      </c>
+      <c r="F70">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
       <c r="A71" s="3">
         <v>46054</v>
       </c>
@@ -4627,6 +5053,12 @@
       </c>
       <c r="D71" s="17">
         <v>26.11</v>
+      </c>
+      <c r="E71">
+        <v>91</v>
+      </c>
+      <c r="F71">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Payroll and Staffing Data Update
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{971CC41A-550D-42BD-B961-B253DB1E5C8E}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5DEC143-0107-4AE3-AC3B-A0C22B10266F}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1687,12 +1687,18 @@
       <c r="A59" s="3">
         <v>46061</v>
       </c>
-      <c r="B59" s="6"/>
+      <c r="B59" s="6">
+        <v>179969.4499999999</v>
+      </c>
       <c r="C59" s="12">
         <v>307344.53999999957</v>
       </c>
-      <c r="D59" s="6"/>
-      <c r="E59" s="17"/>
+      <c r="D59" s="6">
+        <v>29009.63</v>
+      </c>
+      <c r="E59" s="17">
+        <v>0.16119196897028923</v>
+      </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="3"/>
@@ -3114,11 +3120,17 @@
       <c r="B59">
         <v>802</v>
       </c>
+      <c r="C59">
+        <v>665</v>
+      </c>
       <c r="E59" s="3">
         <v>46061</v>
       </c>
       <c r="F59">
         <v>0.97330000000000005</v>
+      </c>
+      <c r="G59">
+        <v>0.72919999999999996</v>
       </c>
     </row>
     <row r="60" spans="1:7">

</xml_diff>

<commit_message>
Payroll and Recruiting Data Update
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5DEC143-0107-4AE3-AC3B-A0C22B10266F}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31541999-B5C4-44F1-9391-7E035BAD4C4A}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="47895" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1701,13 +1701,21 @@
       </c>
     </row>
     <row r="60" spans="1:6">
-      <c r="A60" s="3"/>
-      <c r="B60" s="6"/>
+      <c r="A60" s="3">
+        <v>46068</v>
+      </c>
+      <c r="B60" s="6">
+        <v>194687.86999999956</v>
+      </c>
       <c r="C60" s="12">
         <v>327003.24000000022</v>
       </c>
-      <c r="D60" s="6"/>
-      <c r="E60" s="17"/>
+      <c r="D60" s="6">
+        <v>10413.379999999999</v>
+      </c>
+      <c r="E60" s="17">
+        <v>5.3487564479492343E-2</v>
+      </c>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="3"/>
@@ -3140,11 +3148,17 @@
       <c r="B60">
         <v>794</v>
       </c>
+      <c r="C60">
+        <v>729</v>
+      </c>
       <c r="E60" s="3">
         <v>46068</v>
       </c>
       <c r="F60">
         <v>0.98629999999999995</v>
+      </c>
+      <c r="G60">
+        <v>0.88790000000000002</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -3599,7 +3613,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -5118,6 +5132,26 @@
         <v>265</v>
       </c>
     </row>
+    <row r="73" spans="1:6">
+      <c r="A73" s="3">
+        <v>46068</v>
+      </c>
+      <c r="B73">
+        <v>972</v>
+      </c>
+      <c r="C73">
+        <v>274</v>
+      </c>
+      <c r="D73" s="16">
+        <v>27.24</v>
+      </c>
+      <c r="E73">
+        <v>1615</v>
+      </c>
+      <c r="F73">
+        <v>250</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Payroll Data Update 2-22-26
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://culinarystaffing-my.sharepoint.com/personal/jake_golivestaffing_com/Documents/Documents/GitHub/GoLive_Staffing/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E273DB2-922B-4265-9D33-B56CAC4F8714}"/>
+  <xr:revisionPtr revIDLastSave="93" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C670255-7D8D-45F7-A5E5-EB5D22DDBEB0}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="7845" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -546,13 +546,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F816EB9-28A4-4EE2-B083-40DDC67AF2B4}">
   <dimension ref="A1:F105"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" customWidth="1"/>
+    <col min="1" max="1" width="15.88671875" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="3" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" customWidth="1"/>
+    <col min="5" max="5" width="26.5546875" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1718,13 +1718,21 @@
       </c>
     </row>
     <row r="61" spans="1:6">
-      <c r="A61" s="3"/>
-      <c r="B61" s="6"/>
+      <c r="A61" s="3">
+        <v>46075</v>
+      </c>
+      <c r="B61" s="6">
+        <v>200855.62</v>
+      </c>
       <c r="C61" s="12">
         <v>282217.79999999958</v>
       </c>
-      <c r="D61" s="6"/>
-      <c r="E61" s="17"/>
+      <c r="D61" s="6">
+        <v>18088.34</v>
+      </c>
+      <c r="E61" s="17">
+        <v>9.0056429588577111E-2</v>
+      </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="3"/>
@@ -1953,12 +1961,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AC1FE54-5241-4EDC-8539-E8BDF3481B66}">
   <dimension ref="A1:G105"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1981,7 +1989,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75">
+    <row r="2" spans="1:7" ht="15.6">
       <c r="A2" s="3">
         <v>45662</v>
       </c>
@@ -2001,7 +2009,7 @@
         <v>0.95940000000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75">
+    <row r="3" spans="1:7" ht="15.6">
       <c r="A3" s="3">
         <v>45669</v>
       </c>
@@ -2021,7 +2029,7 @@
         <v>0.9899</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75">
+    <row r="4" spans="1:7" ht="15.6">
       <c r="A4" s="3">
         <v>45676</v>
       </c>
@@ -2041,7 +2049,7 @@
         <v>0.97989999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75">
+    <row r="5" spans="1:7" ht="15.6">
       <c r="A5" s="3">
         <v>45683</v>
       </c>
@@ -2061,7 +2069,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.75">
+    <row r="6" spans="1:7" ht="15.6">
       <c r="A6" s="3">
         <v>45690</v>
       </c>
@@ -2081,7 +2089,7 @@
         <v>0.97460000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75">
+    <row r="7" spans="1:7" ht="15.6">
       <c r="A7" s="3">
         <v>45697</v>
       </c>
@@ -2101,7 +2109,7 @@
         <v>0.97330000000000005</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.75">
+    <row r="8" spans="1:7" ht="15.6">
       <c r="A8" s="3">
         <v>45704</v>
       </c>
@@ -2121,7 +2129,7 @@
         <v>0.98629999999999995</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.75">
+    <row r="9" spans="1:7" ht="15.6">
       <c r="A9" s="3">
         <v>45711</v>
       </c>
@@ -2141,7 +2149,7 @@
         <v>0.98870000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.75">
+    <row r="10" spans="1:7" ht="15.6">
       <c r="A10" s="3">
         <v>45718</v>
       </c>
@@ -2161,7 +2169,7 @@
         <v>0.97619999999999996</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15.75">
+    <row r="11" spans="1:7" ht="15.6">
       <c r="A11" s="3">
         <v>45725</v>
       </c>
@@ -2181,7 +2189,7 @@
         <v>0.98180000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15.75">
+    <row r="12" spans="1:7" ht="15.6">
       <c r="A12" s="3">
         <v>45732</v>
       </c>
@@ -2201,7 +2209,7 @@
         <v>0.98360000000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15.75">
+    <row r="13" spans="1:7" ht="15.6">
       <c r="A13" s="3">
         <v>45739</v>
       </c>
@@ -2221,7 +2229,7 @@
         <v>0.95730000000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.75">
+    <row r="14" spans="1:7" ht="15.6">
       <c r="A14" s="3">
         <v>45746</v>
       </c>
@@ -2241,7 +2249,7 @@
         <v>0.97409999999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="15.75">
+    <row r="15" spans="1:7" ht="15.6">
       <c r="A15" s="3">
         <v>45753</v>
       </c>
@@ -2261,7 +2269,7 @@
         <v>0.97550000000000003</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15.75">
+    <row r="16" spans="1:7" ht="15.6">
       <c r="A16" s="3">
         <v>45760</v>
       </c>
@@ -2281,7 +2289,7 @@
         <v>0.95369999999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.75">
+    <row r="17" spans="1:7" ht="15.6">
       <c r="A17" s="3">
         <v>45767</v>
       </c>
@@ -2301,7 +2309,7 @@
         <v>0.96419999999999995</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.75">
+    <row r="18" spans="1:7" ht="15.6">
       <c r="A18" s="3">
         <v>45774</v>
       </c>
@@ -2321,7 +2329,7 @@
         <v>0.93930000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.75">
+    <row r="19" spans="1:7" ht="15.6">
       <c r="A19" s="3">
         <v>45781</v>
       </c>
@@ -2341,7 +2349,7 @@
         <v>0.94069999999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.75">
+    <row r="20" spans="1:7" ht="15.6">
       <c r="A20" s="3">
         <v>45788</v>
       </c>
@@ -2361,7 +2369,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.75">
+    <row r="21" spans="1:7" ht="15.6">
       <c r="A21" s="3">
         <v>45795</v>
       </c>
@@ -2381,7 +2389,7 @@
         <v>0.93989999999999996</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.75">
+    <row r="22" spans="1:7" ht="15.6">
       <c r="A22" s="3">
         <v>45802</v>
       </c>
@@ -2401,7 +2409,7 @@
         <v>0.95679999999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15.75">
+    <row r="23" spans="1:7" ht="15.6">
       <c r="A23" s="3">
         <v>45809</v>
       </c>
@@ -2421,7 +2429,7 @@
         <v>0.96899999999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.75">
+    <row r="24" spans="1:7" ht="15.6">
       <c r="A24" s="3">
         <v>45816</v>
       </c>
@@ -2441,7 +2449,7 @@
         <v>0.91600000000000004</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.75">
+    <row r="25" spans="1:7" ht="15.6">
       <c r="A25" s="3">
         <v>45823</v>
       </c>
@@ -2461,7 +2469,7 @@
         <v>0.92430000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.75">
+    <row r="26" spans="1:7" ht="15.6">
       <c r="A26" s="3">
         <v>45830</v>
       </c>
@@ -2481,7 +2489,7 @@
         <v>0.96389999999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15.75">
+    <row r="27" spans="1:7" ht="15.6">
       <c r="A27" s="3">
         <v>45837</v>
       </c>
@@ -2501,7 +2509,7 @@
         <v>0.96460000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15.75">
+    <row r="28" spans="1:7" ht="15.6">
       <c r="A28" s="3">
         <v>45844</v>
       </c>
@@ -2521,7 +2529,7 @@
         <v>0.97829999999999995</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15.75">
+    <row r="29" spans="1:7" ht="15.6">
       <c r="A29" s="3">
         <v>45851</v>
       </c>
@@ -2541,7 +2549,7 @@
         <v>0.9738</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.75">
+    <row r="30" spans="1:7" ht="15.6">
       <c r="A30" s="3">
         <v>45858</v>
       </c>
@@ -2561,7 +2569,7 @@
         <v>0.97460000000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15.75">
+    <row r="31" spans="1:7" ht="15.6">
       <c r="A31" s="3">
         <v>45865</v>
       </c>
@@ -2581,7 +2589,7 @@
         <v>0.97160000000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15.75">
+    <row r="32" spans="1:7" ht="15.6">
       <c r="A32" s="3">
         <v>45872</v>
       </c>
@@ -2601,7 +2609,7 @@
         <v>0.95909999999999995</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15.75">
+    <row r="33" spans="1:7" ht="15.6">
       <c r="A33" s="3">
         <v>45879</v>
       </c>
@@ -2621,7 +2629,7 @@
         <v>0.86850000000000005</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15.75">
+    <row r="34" spans="1:7" ht="15.6">
       <c r="A34" s="3">
         <v>45886</v>
       </c>
@@ -2641,7 +2649,7 @@
         <v>0.9395</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15.75">
+    <row r="35" spans="1:7" ht="15.6">
       <c r="A35" s="3">
         <v>45893</v>
       </c>
@@ -2661,7 +2669,7 @@
         <v>0.95920000000000005</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15.75">
+    <row r="36" spans="1:7" ht="15.6">
       <c r="A36" s="3">
         <v>45900</v>
       </c>
@@ -2681,7 +2689,7 @@
         <v>0.97289999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15.75">
+    <row r="37" spans="1:7" ht="15.6">
       <c r="A37" s="3">
         <v>45907</v>
       </c>
@@ -2701,7 +2709,7 @@
         <v>0.92749999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15.75">
+    <row r="38" spans="1:7" ht="15.6">
       <c r="A38" s="3">
         <v>45914</v>
       </c>
@@ -2721,7 +2729,7 @@
         <v>0.92679999999999996</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="15.75">
+    <row r="39" spans="1:7" ht="15.6">
       <c r="A39" s="3">
         <v>45921</v>
       </c>
@@ -2741,7 +2749,7 @@
         <v>0.89119999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="15.75">
+    <row r="40" spans="1:7" ht="15.6">
       <c r="A40" s="3">
         <v>45928</v>
       </c>
@@ -2761,7 +2769,7 @@
         <v>0.93049999999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="15.75">
+    <row r="41" spans="1:7" ht="15.6">
       <c r="A41" s="3">
         <v>45935</v>
       </c>
@@ -2781,7 +2789,7 @@
         <v>0.9264</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.75">
+    <row r="42" spans="1:7" ht="15.6">
       <c r="A42" s="3">
         <v>45942</v>
       </c>
@@ -2801,7 +2809,7 @@
         <v>0.94020000000000004</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15.75">
+    <row r="43" spans="1:7" ht="15.6">
       <c r="A43" s="3">
         <v>45949</v>
       </c>
@@ -2821,7 +2829,7 @@
         <v>0.88719999999999999</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="15.75">
+    <row r="44" spans="1:7" ht="15.6">
       <c r="A44" s="3">
         <v>45956</v>
       </c>
@@ -2841,7 +2849,7 @@
         <v>0.95099999999999996</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="15.75">
+    <row r="45" spans="1:7" ht="15.6">
       <c r="A45" s="3">
         <v>45963</v>
       </c>
@@ -2861,7 +2869,7 @@
         <v>0.95069999999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15.75">
+    <row r="46" spans="1:7" ht="15.6">
       <c r="A46" s="3">
         <v>45970</v>
       </c>
@@ -2881,7 +2889,7 @@
         <v>0.95689999999999997</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="15.75">
+    <row r="47" spans="1:7" ht="15.6">
       <c r="A47" s="3">
         <v>45977</v>
       </c>
@@ -2901,7 +2909,7 @@
         <v>0.87290000000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15.75">
+    <row r="48" spans="1:7" ht="15.6">
       <c r="A48" s="3">
         <v>45984</v>
       </c>
@@ -2921,7 +2929,7 @@
         <v>0.95269999999999999</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="15.75">
+    <row r="49" spans="1:7" ht="15.6">
       <c r="A49" s="3">
         <v>45991</v>
       </c>
@@ -2941,7 +2949,7 @@
         <v>0.97119999999999995</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="15.75">
+    <row r="50" spans="1:7" ht="15.6">
       <c r="A50" s="3">
         <v>45998</v>
       </c>
@@ -2961,7 +2969,7 @@
         <v>0.95509999999999995</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="15.75">
+    <row r="51" spans="1:7" ht="15.6">
       <c r="A51" s="3">
         <v>46005</v>
       </c>
@@ -2981,7 +2989,7 @@
         <v>0.91969999999999996</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="15.75">
+    <row r="52" spans="1:7" ht="15.6">
       <c r="A52" s="3">
         <v>46012</v>
       </c>
@@ -3001,7 +3009,7 @@
         <v>0.96120000000000005</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="15.75">
+    <row r="53" spans="1:7" ht="15.6">
       <c r="A53" s="3">
         <v>46019</v>
       </c>
@@ -3168,11 +3176,17 @@
       <c r="B61">
         <v>703</v>
       </c>
+      <c r="C61">
+        <v>751</v>
+      </c>
       <c r="E61" s="3">
         <v>46075</v>
       </c>
       <c r="F61">
         <v>0.98870000000000002</v>
+      </c>
+      <c r="G61">
+        <v>0.94350000000000001</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -3613,15 +3627,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
-  <dimension ref="A1:F74"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:F75"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.6640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -5172,6 +5186,9 @@
         <v>204</v>
       </c>
     </row>
+    <row r="75" spans="1:6">
+      <c r="A75" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data update and lunch break fix
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C670255-7D8D-45F7-A5E5-EB5D22DDBEB0}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A787DF0-7E92-47C5-A46E-CD28FD539345}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="47895" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -226,6 +226,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -546,13 +550,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F816EB9-28A4-4EE2-B083-40DDC67AF2B4}">
   <dimension ref="A1:F105"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.88671875" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="20.109375" customWidth="1"/>
-    <col min="5" max="5" width="26.5546875" customWidth="1"/>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="26.5703125" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1735,13 +1739,21 @@
       </c>
     </row>
     <row r="62" spans="1:6">
-      <c r="A62" s="3"/>
-      <c r="B62" s="6"/>
+      <c r="A62" s="3">
+        <v>46082</v>
+      </c>
+      <c r="B62" s="6">
+        <v>252257.11999999889</v>
+      </c>
       <c r="C62" s="12">
         <v>406848.86999999994</v>
       </c>
-      <c r="D62" s="6"/>
-      <c r="E62" s="17"/>
+      <c r="D62" s="6">
+        <v>62988.69</v>
+      </c>
+      <c r="E62" s="17">
+        <v>0.2497003454253354</v>
+      </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="3"/>
@@ -1961,12 +1973,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AC1FE54-5241-4EDC-8539-E8BDF3481B66}">
   <dimension ref="A1:G105"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1989,7 +2001,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.6">
+    <row r="2" spans="1:7" ht="15.75">
       <c r="A2" s="3">
         <v>45662</v>
       </c>
@@ -2009,7 +2021,7 @@
         <v>0.95940000000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.6">
+    <row r="3" spans="1:7" ht="15.75">
       <c r="A3" s="3">
         <v>45669</v>
       </c>
@@ -2029,7 +2041,7 @@
         <v>0.9899</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.6">
+    <row r="4" spans="1:7" ht="15.75">
       <c r="A4" s="3">
         <v>45676</v>
       </c>
@@ -2049,7 +2061,7 @@
         <v>0.97989999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.6">
+    <row r="5" spans="1:7" ht="15.75">
       <c r="A5" s="3">
         <v>45683</v>
       </c>
@@ -2069,7 +2081,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.6">
+    <row r="6" spans="1:7" ht="15.75">
       <c r="A6" s="3">
         <v>45690</v>
       </c>
@@ -2089,7 +2101,7 @@
         <v>0.97460000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.6">
+    <row r="7" spans="1:7" ht="15.75">
       <c r="A7" s="3">
         <v>45697</v>
       </c>
@@ -2109,7 +2121,7 @@
         <v>0.97330000000000005</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.6">
+    <row r="8" spans="1:7" ht="15.75">
       <c r="A8" s="3">
         <v>45704</v>
       </c>
@@ -2129,7 +2141,7 @@
         <v>0.98629999999999995</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.6">
+    <row r="9" spans="1:7" ht="15.75">
       <c r="A9" s="3">
         <v>45711</v>
       </c>
@@ -2149,7 +2161,7 @@
         <v>0.98870000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.6">
+    <row r="10" spans="1:7" ht="15.75">
       <c r="A10" s="3">
         <v>45718</v>
       </c>
@@ -2169,7 +2181,7 @@
         <v>0.97619999999999996</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15.6">
+    <row r="11" spans="1:7" ht="15.75">
       <c r="A11" s="3">
         <v>45725</v>
       </c>
@@ -2189,7 +2201,7 @@
         <v>0.98180000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15.6">
+    <row r="12" spans="1:7" ht="15.75">
       <c r="A12" s="3">
         <v>45732</v>
       </c>
@@ -2209,7 +2221,7 @@
         <v>0.98360000000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15.6">
+    <row r="13" spans="1:7" ht="15.75">
       <c r="A13" s="3">
         <v>45739</v>
       </c>
@@ -2229,7 +2241,7 @@
         <v>0.95730000000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.6">
+    <row r="14" spans="1:7" ht="15.75">
       <c r="A14" s="3">
         <v>45746</v>
       </c>
@@ -2249,7 +2261,7 @@
         <v>0.97409999999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="15.6">
+    <row r="15" spans="1:7" ht="15.75">
       <c r="A15" s="3">
         <v>45753</v>
       </c>
@@ -2269,7 +2281,7 @@
         <v>0.97550000000000003</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15.6">
+    <row r="16" spans="1:7" ht="15.75">
       <c r="A16" s="3">
         <v>45760</v>
       </c>
@@ -2289,7 +2301,7 @@
         <v>0.95369999999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.6">
+    <row r="17" spans="1:7" ht="15.75">
       <c r="A17" s="3">
         <v>45767</v>
       </c>
@@ -2309,7 +2321,7 @@
         <v>0.96419999999999995</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.6">
+    <row r="18" spans="1:7" ht="15.75">
       <c r="A18" s="3">
         <v>45774</v>
       </c>
@@ -2329,7 +2341,7 @@
         <v>0.93930000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.6">
+    <row r="19" spans="1:7" ht="15.75">
       <c r="A19" s="3">
         <v>45781</v>
       </c>
@@ -2349,7 +2361,7 @@
         <v>0.94069999999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.6">
+    <row r="20" spans="1:7" ht="15.75">
       <c r="A20" s="3">
         <v>45788</v>
       </c>
@@ -2369,7 +2381,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.6">
+    <row r="21" spans="1:7" ht="15.75">
       <c r="A21" s="3">
         <v>45795</v>
       </c>
@@ -2389,7 +2401,7 @@
         <v>0.93989999999999996</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.6">
+    <row r="22" spans="1:7" ht="15.75">
       <c r="A22" s="3">
         <v>45802</v>
       </c>
@@ -2409,7 +2421,7 @@
         <v>0.95679999999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15.6">
+    <row r="23" spans="1:7" ht="15.75">
       <c r="A23" s="3">
         <v>45809</v>
       </c>
@@ -2429,7 +2441,7 @@
         <v>0.96899999999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.6">
+    <row r="24" spans="1:7" ht="15.75">
       <c r="A24" s="3">
         <v>45816</v>
       </c>
@@ -2449,7 +2461,7 @@
         <v>0.91600000000000004</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.6">
+    <row r="25" spans="1:7" ht="15.75">
       <c r="A25" s="3">
         <v>45823</v>
       </c>
@@ -2469,7 +2481,7 @@
         <v>0.92430000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.6">
+    <row r="26" spans="1:7" ht="15.75">
       <c r="A26" s="3">
         <v>45830</v>
       </c>
@@ -2489,7 +2501,7 @@
         <v>0.96389999999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15.6">
+    <row r="27" spans="1:7" ht="15.75">
       <c r="A27" s="3">
         <v>45837</v>
       </c>
@@ -2509,7 +2521,7 @@
         <v>0.96460000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15.6">
+    <row r="28" spans="1:7" ht="15.75">
       <c r="A28" s="3">
         <v>45844</v>
       </c>
@@ -2529,7 +2541,7 @@
         <v>0.97829999999999995</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15.6">
+    <row r="29" spans="1:7" ht="15.75">
       <c r="A29" s="3">
         <v>45851</v>
       </c>
@@ -2549,7 +2561,7 @@
         <v>0.9738</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.6">
+    <row r="30" spans="1:7" ht="15.75">
       <c r="A30" s="3">
         <v>45858</v>
       </c>
@@ -2569,7 +2581,7 @@
         <v>0.97460000000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15.6">
+    <row r="31" spans="1:7" ht="15.75">
       <c r="A31" s="3">
         <v>45865</v>
       </c>
@@ -2589,7 +2601,7 @@
         <v>0.97160000000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15.6">
+    <row r="32" spans="1:7" ht="15.75">
       <c r="A32" s="3">
         <v>45872</v>
       </c>
@@ -2609,7 +2621,7 @@
         <v>0.95909999999999995</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15.6">
+    <row r="33" spans="1:7" ht="15.75">
       <c r="A33" s="3">
         <v>45879</v>
       </c>
@@ -2629,7 +2641,7 @@
         <v>0.86850000000000005</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15.6">
+    <row r="34" spans="1:7" ht="15.75">
       <c r="A34" s="3">
         <v>45886</v>
       </c>
@@ -2649,7 +2661,7 @@
         <v>0.9395</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15.6">
+    <row r="35" spans="1:7" ht="15.75">
       <c r="A35" s="3">
         <v>45893</v>
       </c>
@@ -2669,7 +2681,7 @@
         <v>0.95920000000000005</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15.6">
+    <row r="36" spans="1:7" ht="15.75">
       <c r="A36" s="3">
         <v>45900</v>
       </c>
@@ -2689,7 +2701,7 @@
         <v>0.97289999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15.6">
+    <row r="37" spans="1:7" ht="15.75">
       <c r="A37" s="3">
         <v>45907</v>
       </c>
@@ -2709,7 +2721,7 @@
         <v>0.92749999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15.6">
+    <row r="38" spans="1:7" ht="15.75">
       <c r="A38" s="3">
         <v>45914</v>
       </c>
@@ -2729,7 +2741,7 @@
         <v>0.92679999999999996</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="15.6">
+    <row r="39" spans="1:7" ht="15.75">
       <c r="A39" s="3">
         <v>45921</v>
       </c>
@@ -2749,7 +2761,7 @@
         <v>0.89119999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="15.6">
+    <row r="40" spans="1:7" ht="15.75">
       <c r="A40" s="3">
         <v>45928</v>
       </c>
@@ -2769,7 +2781,7 @@
         <v>0.93049999999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="15.6">
+    <row r="41" spans="1:7" ht="15.75">
       <c r="A41" s="3">
         <v>45935</v>
       </c>
@@ -2789,7 +2801,7 @@
         <v>0.9264</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.6">
+    <row r="42" spans="1:7" ht="15.75">
       <c r="A42" s="3">
         <v>45942</v>
       </c>
@@ -2809,7 +2821,7 @@
         <v>0.94020000000000004</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15.6">
+    <row r="43" spans="1:7" ht="15.75">
       <c r="A43" s="3">
         <v>45949</v>
       </c>
@@ -2829,7 +2841,7 @@
         <v>0.88719999999999999</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="15.6">
+    <row r="44" spans="1:7" ht="15.75">
       <c r="A44" s="3">
         <v>45956</v>
       </c>
@@ -2849,7 +2861,7 @@
         <v>0.95099999999999996</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="15.6">
+    <row r="45" spans="1:7" ht="15.75">
       <c r="A45" s="3">
         <v>45963</v>
       </c>
@@ -2869,7 +2881,7 @@
         <v>0.95069999999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15.6">
+    <row r="46" spans="1:7" ht="15.75">
       <c r="A46" s="3">
         <v>45970</v>
       </c>
@@ -2889,7 +2901,7 @@
         <v>0.95689999999999997</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="15.6">
+    <row r="47" spans="1:7" ht="15.75">
       <c r="A47" s="3">
         <v>45977</v>
       </c>
@@ -2909,7 +2921,7 @@
         <v>0.87290000000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15.6">
+    <row r="48" spans="1:7" ht="15.75">
       <c r="A48" s="3">
         <v>45984</v>
       </c>
@@ -2929,7 +2941,7 @@
         <v>0.95269999999999999</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="15.6">
+    <row r="49" spans="1:7" ht="15.75">
       <c r="A49" s="3">
         <v>45991</v>
       </c>
@@ -2949,7 +2961,7 @@
         <v>0.97119999999999995</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="15.6">
+    <row r="50" spans="1:7" ht="15.75">
       <c r="A50" s="3">
         <v>45998</v>
       </c>
@@ -2969,7 +2981,7 @@
         <v>0.95509999999999995</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="15.6">
+    <row r="51" spans="1:7" ht="15.75">
       <c r="A51" s="3">
         <v>46005</v>
       </c>
@@ -2989,7 +3001,7 @@
         <v>0.91969999999999996</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="15.6">
+    <row r="52" spans="1:7" ht="15.75">
       <c r="A52" s="3">
         <v>46012</v>
       </c>
@@ -3009,7 +3021,7 @@
         <v>0.96120000000000005</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="15.6">
+    <row r="53" spans="1:7" ht="15.75">
       <c r="A53" s="3">
         <v>46019</v>
       </c>
@@ -3196,11 +3208,17 @@
       <c r="B62">
         <v>986</v>
       </c>
+      <c r="C62">
+        <v>966</v>
+      </c>
       <c r="E62" s="3">
         <v>46082</v>
       </c>
       <c r="F62">
         <v>0.97619999999999996</v>
+      </c>
+      <c r="G62">
+        <v>0.9113</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -3628,14 +3646,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
   <dimension ref="A1:F75"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.6640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.7109375" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -5187,7 +5205,24 @@
       </c>
     </row>
     <row r="75" spans="1:6">
-      <c r="A75" s="3"/>
+      <c r="A75" s="3">
+        <v>46082</v>
+      </c>
+      <c r="B75">
+        <v>995</v>
+      </c>
+      <c r="C75">
+        <v>363</v>
+      </c>
+      <c r="D75" s="16">
+        <v>36.479999999999997</v>
+      </c>
+      <c r="E75">
+        <v>1043</v>
+      </c>
+      <c r="F75">
+        <v>277</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
API and Recruiting Data Update
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A787DF0-7E92-47C5-A46E-CD28FD539345}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69B82AAD-F29F-412C-9BB6-BBB682512318}"/>
   <bookViews>
-    <workbookView xWindow="47895" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="52065" yWindow="0" windowWidth="15240" windowHeight="20985" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -3645,7 +3645,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -5224,6 +5224,26 @@
         <v>277</v>
       </c>
     </row>
+    <row r="76" spans="1:6">
+      <c r="A76" s="3">
+        <v>46089</v>
+      </c>
+      <c r="B76">
+        <v>1010</v>
+      </c>
+      <c r="C76">
+        <v>381</v>
+      </c>
+      <c r="D76" s="16">
+        <v>37.72</v>
+      </c>
+      <c r="E76">
+        <v>472</v>
+      </c>
+      <c r="F76">
+        <v>119</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Staffing Data Update and Recruiting Map
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="115" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69B82AAD-F29F-412C-9BB6-BBB682512318}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8318A915-C098-41E1-8094-17CC351D77CE}"/>
   <bookViews>
-    <workbookView xWindow="52065" yWindow="0" windowWidth="15240" windowHeight="20985" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1756,13 +1756,21 @@
       </c>
     </row>
     <row r="63" spans="1:6">
-      <c r="A63" s="3"/>
-      <c r="B63" s="6"/>
+      <c r="A63" s="3">
+        <v>46089</v>
+      </c>
+      <c r="B63" s="6">
+        <v>306206.7299999987</v>
+      </c>
       <c r="C63" s="12">
         <v>492946.42999999959</v>
       </c>
-      <c r="D63" s="6"/>
-      <c r="E63" s="17"/>
+      <c r="D63" s="6">
+        <v>120206.45</v>
+      </c>
+      <c r="E63" s="17">
+        <v>0.39256632275848574</v>
+      </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="3"/>
@@ -3228,11 +3236,17 @@
       <c r="B63">
         <v>864</v>
       </c>
+      <c r="C63">
+        <v>1120</v>
+      </c>
       <c r="E63" s="3">
         <v>46089</v>
       </c>
       <c r="F63">
         <v>0.98180000000000001</v>
+      </c>
+      <c r="G63">
+        <v>0.81930000000000003</v>
       </c>
     </row>
     <row r="64" spans="1:7">

</xml_diff>

<commit_message>
Data update and Payroll Notes
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="146" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{338AE5D0-108F-48E6-93A8-8CEE928F811F}"/>
+  <xr:revisionPtr revIDLastSave="153" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BA5A93E-DD14-436E-BD3B-1C2520743E16}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="36315" yWindow="1575" windowWidth="21600" windowHeight="12645" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1793,12 +1793,18 @@
       <c r="A65" s="3">
         <v>46103</v>
       </c>
-      <c r="B65" s="6"/>
+      <c r="B65" s="6">
+        <v>193573.41999999993</v>
+      </c>
       <c r="C65" s="12">
         <v>375603.12999999931</v>
       </c>
-      <c r="D65" s="6"/>
-      <c r="E65" s="17"/>
+      <c r="D65" s="6">
+        <v>19608.54</v>
+      </c>
+      <c r="E65" s="17">
+        <v>0.10129768849462911</v>
+      </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" s="3"/>
@@ -3292,21 +3298,27 @@
         <v>0.85150000000000003</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:7">
       <c r="A65" s="3">
         <v>46103</v>
       </c>
       <c r="B65">
         <v>1010</v>
       </c>
+      <c r="C65">
+        <v>741</v>
+      </c>
       <c r="E65" s="3">
         <v>46103</v>
       </c>
       <c r="F65">
         <v>0.95730000000000004</v>
       </c>
-    </row>
-    <row r="66" spans="1:6">
+      <c r="G65">
+        <v>0.87180000000000002</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7">
       <c r="A66" s="3">
         <v>46110</v>
       </c>
@@ -3320,7 +3332,7 @@
         <v>0.97409999999999997</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:7">
       <c r="A67" s="3">
         <v>46117</v>
       </c>
@@ -3334,7 +3346,7 @@
         <v>0.97550000000000003</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:7">
       <c r="A68" s="3">
         <v>46124</v>
       </c>
@@ -3348,7 +3360,7 @@
         <v>0.95369999999999999</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:7">
       <c r="A69" s="3">
         <v>46131</v>
       </c>
@@ -3362,7 +3374,7 @@
         <v>0.96419999999999995</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:7">
       <c r="A70" s="3">
         <v>46138</v>
       </c>
@@ -3376,7 +3388,7 @@
         <v>0.93930000000000002</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:7">
       <c r="A71" s="3">
         <v>46145</v>
       </c>
@@ -3390,7 +3402,7 @@
         <v>0.94069999999999998</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:7">
       <c r="A72" s="3">
         <v>46152</v>
       </c>
@@ -3404,7 +3416,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:7">
       <c r="A73" s="3">
         <v>46159</v>
       </c>
@@ -3418,7 +3430,7 @@
         <v>0.93989999999999996</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:7">
       <c r="A74" s="3">
         <v>46166</v>
       </c>
@@ -3432,7 +3444,7 @@
         <v>0.95679999999999998</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:7">
       <c r="A75" s="3"/>
       <c r="B75">
         <v>688</v>
@@ -3441,7 +3453,7 @@
         <v>0.96899999999999997</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:7">
       <c r="B76">
         <v>884</v>
       </c>
@@ -3449,7 +3461,7 @@
         <v>0.91600000000000004</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:7">
       <c r="B77">
         <v>745</v>
       </c>
@@ -3457,7 +3469,7 @@
         <v>0.92430000000000001</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:7">
       <c r="B78">
         <v>668</v>
       </c>
@@ -3465,7 +3477,7 @@
         <v>0.96389999999999998</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:7">
       <c r="B79">
         <v>763</v>
       </c>
@@ -3473,7 +3485,7 @@
         <v>0.96460000000000001</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:7">
       <c r="B80">
         <v>497</v>
       </c>

</xml_diff>

<commit_message>
Adding Notes analysis to employee dashboard
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="153" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BA5A93E-DD14-436E-BD3B-1C2520743E16}"/>
+  <xr:revisionPtr revIDLastSave="167" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59015AD8-29AE-4FDC-A2C9-0F00DFCDFAF7}"/>
   <bookViews>
-    <workbookView xWindow="36315" yWindow="1575" windowWidth="21600" windowHeight="12645" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1807,13 +1807,21 @@
       </c>
     </row>
     <row r="66" spans="1:5">
-      <c r="A66" s="3"/>
-      <c r="B66" s="6"/>
+      <c r="A66" s="3">
+        <v>46110</v>
+      </c>
+      <c r="B66" s="6">
+        <v>218457.35</v>
+      </c>
       <c r="C66" s="12">
         <v>340411.14000000025</v>
       </c>
-      <c r="D66" s="6"/>
-      <c r="E66" s="17"/>
+      <c r="D66" s="6">
+        <v>17373.64</v>
+      </c>
+      <c r="E66" s="17">
+        <v>7.9528750119874647E-2</v>
+      </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="3"/>
@@ -3325,11 +3333,17 @@
       <c r="B66">
         <v>901</v>
       </c>
+      <c r="C66">
+        <v>834</v>
+      </c>
       <c r="E66" s="3">
         <v>46110</v>
       </c>
       <c r="F66">
         <v>0.97409999999999997</v>
+      </c>
+      <c r="G66">
+        <v>0.92869999999999997</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -3700,7 +3714,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -5339,6 +5353,26 @@
         <v>104</v>
       </c>
     </row>
+    <row r="79" spans="1:6">
+      <c r="A79" s="3">
+        <v>46110</v>
+      </c>
+      <c r="B79">
+        <v>1024</v>
+      </c>
+      <c r="C79">
+        <v>321</v>
+      </c>
+      <c r="D79" s="16">
+        <v>31.35</v>
+      </c>
+      <c r="E79">
+        <v>469</v>
+      </c>
+      <c r="F79">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Render bug fix and recruiting data upload
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="167" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59015AD8-29AE-4FDC-A2C9-0F00DFCDFAF7}"/>
+  <xr:revisionPtr revIDLastSave="175" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E11489C-AE06-4282-931A-C53C7F6367EB}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1824,7 +1824,9 @@
       </c>
     </row>
     <row r="67" spans="1:5">
-      <c r="A67" s="3"/>
+      <c r="A67" s="3">
+        <v>46117</v>
+      </c>
       <c r="B67" s="6"/>
       <c r="C67" s="12">
         <v>273530.54999999987</v>
@@ -3714,7 +3716,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -5373,6 +5375,26 @@
         <v>84</v>
       </c>
     </row>
+    <row r="80" spans="1:6">
+      <c r="A80" s="3">
+        <v>46117</v>
+      </c>
+      <c r="B80">
+        <v>999</v>
+      </c>
+      <c r="C80">
+        <v>293</v>
+      </c>
+      <c r="D80" s="16">
+        <v>29.33</v>
+      </c>
+      <c r="E80">
+        <v>822</v>
+      </c>
+      <c r="F80">
+        <v>209</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Sick Pay email and Basic Client report
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="305" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCA471B5-FEEA-40FD-9519-D0E0610775A7}"/>
+  <xr:revisionPtr revIDLastSave="307" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F74492B1-9C57-4E44-B419-78ADD0EE6340}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-4560" windowWidth="38640" windowHeight="21120" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="3570" yWindow="1245" windowWidth="21600" windowHeight="12645" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -1963,7 +1963,9 @@
       </c>
     </row>
     <row r="75" spans="1:5">
-      <c r="A75" s="3"/>
+      <c r="A75" s="3">
+        <v>46173</v>
+      </c>
       <c r="B75" s="6"/>
       <c r="C75" s="12">
         <v>265417.39000000007</v>
@@ -3858,7 +3860,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C4474F-08DB-44F2-9F06-11762EAF8D82}">
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -5677,6 +5679,11 @@
         <v>205</v>
       </c>
     </row>
+    <row r="88" spans="1:6">
+      <c r="A88" s="3">
+        <v>46173</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Order with Change Capability
</commit_message>
<xml_diff>
--- a/Sales and Staffing Charts.xlsx
+++ b/Sales and Staffing Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="307" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F74492B1-9C57-4E44-B419-78ADD0EE6340}"/>
+  <xr:revisionPtr revIDLastSave="309" documentId="13_ncr:1_{1D637CDB-FF44-4AB8-99D5-2902FDA30D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2F2C0E1-4D60-43E6-8FE2-1A5DB5688184}"/>
   <bookViews>
-    <workbookView xWindow="3570" yWindow="1245" windowWidth="21600" windowHeight="12645" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{A3B2B6D9-7C24-445E-A372-57A39B7AE13F}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -5683,6 +5683,12 @@
       <c r="A88" s="3">
         <v>46173</v>
       </c>
+      <c r="E88">
+        <v>755</v>
+      </c>
+      <c r="F88">
+        <v>175</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>